<commit_message>
Denominator for lipid claim; eQTLGen-specific wording; protein-coding terminology; title
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dzcr1HX3pctdT6vYSvzwEH
</commit_message>
<xml_diff>
--- a/manuscript_prep/manuscript/display/recovery_tables.xlsx
+++ b/manuscript_prep/manuscript/display/recovery_tables.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,7 +632,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NO CURRENTLY MARKETED DRUG FOUND; discontinued: mipomersen (FDA discontinued; EMA refused)</t>
+          <t>No currently marketed drug found; discontinued: mipomersen (FDA discontinued; EMA refused)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Skin Sun Exposed Lower leg (4.6×10⁻⁵⁸); Skin Not Sun Exposed Suprapubic (2.3×10⁻³⁵); Heart Left Ventricle* (1.1×10⁻³⁰); Adipose Subcutaneous (4.9×10⁻²⁹); Nerve Tibial (8.4×10⁻¹⁶); Heart Atrial Appendage* (1.1×10⁻¹¹); Artery Tibial* (8×10⁻¹¹); Esophagus Gastroesophageal Junction (6.9×10⁻⁰⁹); Esophagus Muscularis (1.1×10⁻⁰⁸)</t>
+          <t>Skin Sun Exposed Lower leg (4.6×10⁻⁵⁸); Skin Not Sun Exposed Suprapubic (2.3×10⁻³⁵); Heart Left Ventricle* (1.1×10⁻³⁰); Adipose Subcutaneous (4.9×10⁻²⁹); Nerve Tibial (8.4×10⁻¹⁶); Heart Atrial Appendage* (1.1×10⁻¹¹); Artery Tibial* (8×10⁻¹¹); Esophagus Gastroesophageal Junction (6.9×10⁻⁹); Esophagus Muscularis (1.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Artery Tibial* (3.3×10⁻¹⁵); Brain Cerebellum (2×10⁻¹²); Testis (1.1×10⁻⁰⁹)</t>
+          <t>Artery Tibial* (3.3×10⁻¹⁵); Brain Cerebellum (2×10⁻¹²); Testis (1.1×10⁻⁹)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Skin Sun Exposed Lower leg (4.3×10⁻²⁴); Ovary (1.5×10⁻¹²); Skin Not Sun Exposed Suprapubic (1.4×10⁻¹¹); Testis (5.9×10⁻¹¹); Brain Cortex (1.6×10⁻⁰⁸)</t>
+          <t>Skin Sun Exposed Lower leg (4.3×10⁻²⁴); Ovary (1.5×10⁻¹²); Skin Not Sun Exposed Suprapubic (1.4×10⁻¹¹); Testis (5.9×10⁻¹¹); Brain Cortex (1.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Thyroid (8.5×10⁻¹⁸); Spleen (4.7×10⁻¹⁴); Nerve Tibial (1.8×10⁻⁰⁹)</t>
+          <t>Thyroid (8.5×10⁻¹⁸); Spleen (4.7×10⁻¹⁴); Nerve Tibial (1.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1318,6 +1318,13 @@
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
+        <is>
+          <t>P values below 1×10⁻³⁰⁰ are derived from the −log10 P reported in the source table, rounded to the nearest power of 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>'Approved' in this study means ever approved by the FDA or the EMA for a cardiovascular indication; the cardiovascular indication is taken from ChEMBL and the approval record from the two agencies' databases.</t>
         </is>
@@ -2081,7 +2088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2874,6 +2881,13 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>A target is counted in every indication area in which it has a programme, so area rows do not sum to the total. Percentages are of the row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Never-assayed counts include microRNA and mitochondrial genes, which no plasma protein panel can measure (9 and 2 overall; 4 and 1 among heart failure and cardiomyopathy targets), so they exceed the protein-coding counts given in the text.</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3138,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Thyroid (3.5×10⁻⁹⁵); Muscle_Skeletal (2.6×10⁻⁸⁵); Skin_Sun_Exposed_Lower_leg (1.4×10⁻⁵⁶); Artery_Aorta (1.1×10⁻⁵²); Artery_Tibial (1.4×10⁻⁴⁸); Skin_Not_Sun_Exposed_Suprapubic (6.8×10⁻⁴¹); Heart_Left_Ventricle (2.3×10⁻⁴⁰); Nerve_Tibial (1.3×10⁻³⁷); Heart_Atrial_Appendage (1.4×10⁻³⁷); Adipose_Subcutaneous (9.4×10⁻³¹); Adipose_Visceral_Omentum (1.9×10⁻²⁵); Artery_Coronary (2.1×10⁻²³); Brain_Cerebellum (1.5×10⁻²¹); Breast_Mammary_Tissue (8.5×10⁻²⁰); Esophagus_Gastroesophageal_Junction (8.8×10⁻¹⁹); Brain_Putamen_basal_ganglia (8.7×10⁻¹⁷); Colon_Sigmoid (2.7×10⁻¹⁶); Brain_Nucleus_accumbens_basal_ganglia (6.3×10⁻¹⁶); Brain_Caudate_basal_ganglia (7.9×10⁻¹⁶); Lung (2.4×10⁻¹⁵); Brain_Hypothalamus (1.1×10⁻¹⁴); Brain_Substantia_nigra (4.3×10⁻¹⁴); Brain_Cerebellar_Hemisphere (6.3×10⁻¹⁴); Brain_Anterior_cingulate_cortex_BA24 (1×10⁻¹³); Testis (4.9×10⁻¹³); Prostate (1×10⁻¹²); Brain_Frontal_Cortex_BA9 (2.3×10⁻¹²); Colon_Transverse (1.4×10⁻¹¹); Stomach (1.9×10⁻¹¹); Esophagus_Mucosa (4.5×10⁻¹¹); Brain_Cortex (7×10⁻¹¹); Brain_Hippocampus (1.6×10⁻¹⁰); Esophagus_Muscularis (3.6×10⁻⁰⁸)</t>
+          <t>Thyroid (3.5×10⁻⁹⁵); Muscle_Skeletal (2.6×10⁻⁸⁵); Skin_Sun_Exposed_Lower_leg (1.4×10⁻⁵⁶); Artery_Aorta (1.1×10⁻⁵²); Artery_Tibial (1.4×10⁻⁴⁸); Skin_Not_Sun_Exposed_Suprapubic (6.8×10⁻⁴¹); Heart_Left_Ventricle (2.3×10⁻⁴⁰); Nerve_Tibial (1.3×10⁻³⁷); Heart_Atrial_Appendage (1.4×10⁻³⁷); Adipose_Subcutaneous (9.4×10⁻³¹); Adipose_Visceral_Omentum (1.9×10⁻²⁵); Artery_Coronary (2.1×10⁻²³); Brain_Cerebellum (1.5×10⁻²¹); Breast_Mammary_Tissue (8.5×10⁻²⁰); Esophagus_Gastroesophageal_Junction (8.8×10⁻¹⁹); Brain_Putamen_basal_ganglia (8.7×10⁻¹⁷); Colon_Sigmoid (2.7×10⁻¹⁶); Brain_Nucleus_accumbens_basal_ganglia (6.3×10⁻¹⁶); Brain_Caudate_basal_ganglia (7.9×10⁻¹⁶); Lung (2.4×10⁻¹⁵); Brain_Hypothalamus (1.1×10⁻¹⁴); Brain_Substantia_nigra (4.3×10⁻¹⁴); Brain_Cerebellar_Hemisphere (6.3×10⁻¹⁴); Brain_Anterior_cingulate_cortex_BA24 (1×10⁻¹³); Testis (4.9×10⁻¹³); Prostate (1×10⁻¹²); Brain_Frontal_Cortex_BA9 (2.3×10⁻¹²); Colon_Transverse (1.4×10⁻¹¹); Stomach (1.9×10⁻¹¹); Esophagus_Mucosa (4.5×10⁻¹¹); Brain_Cortex (7×10⁻¹¹); Brain_Hippocampus (1.6×10⁻¹⁰); Esophagus_Muscularis (3.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -3232,7 +3246,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Adrenal_Gland (3.4×10⁻¹⁶); Brain_Nucleus_accumbens_basal_ganglia (3.4×10⁻¹²); Brain_Caudate_basal_ganglia (1.7×10⁻⁰⁹); Artery_Tibial (4.8×10⁻⁰⁹)</t>
+          <t>Adrenal_Gland (3.4×10⁻¹⁶); Brain_Nucleus_accumbens_basal_ganglia (3.4×10⁻¹²); Brain_Caudate_basal_ganglia (1.7×10⁻⁹); Artery_Tibial (4.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -3344,7 +3358,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Thyroid (6.9×10⁻³⁸); Cells_Cultured_fibroblasts (4.2×10⁻¹⁸); Lung (2.9×10⁻¹⁵); Artery_Tibial (9.3×10⁻¹³); Skin_Sun_Exposed_Lower_leg (5.1×10⁻¹¹); Nerve_Tibial (2.4×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (4×10⁻¹⁰); Esophagus_Mucosa (2.5×10⁻⁰⁹); Spleen (8.8×10⁻⁰⁹); Adipose_Subcutaneous (1.6×10⁻⁰⁸); Esophagus_Muscularis (2.4×10⁻⁰⁸)</t>
+          <t>Thyroid (6.9×10⁻³⁸); Cells_Cultured_fibroblasts (4.2×10⁻¹⁸); Lung (2.9×10⁻¹⁵); Artery_Tibial (9.3×10⁻¹³); Skin_Sun_Exposed_Lower_leg (5.1×10⁻¹¹); Nerve_Tibial (2.4×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (4×10⁻¹⁰); Esophagus_Mucosa (2.5×10⁻⁹); Spleen (8.8×10⁻⁹); Adipose_Subcutaneous (1.6×10⁻⁸); Esophagus_Muscularis (2.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -3456,7 +3470,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Brain_Frontal_Cortex_BA9 (1.4×10⁻¹⁷); Nerve_Tibial (3.3×10⁻¹⁷); Brain_Cortex (8.9×10⁻¹⁷); Brain_Nucleus_accumbens_basal_ganglia (3.2×10⁻¹⁶); Brain_Caudate_basal_ganglia (6.3×10⁻¹³); Brain_Putamen_basal_ganglia (3.6×10⁻¹¹); Brain_Cerebellum (4.3×10⁻¹⁰); Artery_Tibial (6×10⁻¹⁰); Brain_Anterior_cingulate_cortex_BA24 (7.1×10⁻⁰⁹); Brain_Hypothalamus (2.5×10⁻⁰⁸)</t>
+          <t>Brain_Frontal_Cortex_BA9 (1.4×10⁻¹⁷); Nerve_Tibial (3.3×10⁻¹⁷); Brain_Cortex (8.9×10⁻¹⁷); Brain_Nucleus_accumbens_basal_ganglia (3.2×10⁻¹⁶); Brain_Caudate_basal_ganglia (6.3×10⁻¹³); Brain_Putamen_basal_ganglia (3.6×10⁻¹¹); Brain_Cerebellum (4.3×10⁻¹⁰); Artery_Tibial (6×10⁻¹⁰); Brain_Anterior_cingulate_cortex_BA24 (7.1×10⁻⁹); Brain_Hypothalamus (2.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -3576,7 +3590,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Artery_Aorta (1.3×10⁻⁴⁷); Thyroid (5.7×10⁻⁴³); Artery_Tibial (2.2×10⁻⁴²); Nerve_Tibial (5×10⁻⁴²); Adipose_Subcutaneous (6.5×10⁻²⁴); Skin_Sun_Exposed_Lower_leg (8×10⁻²²); Heart_Atrial_Appendage (9.2×10⁻²²); Liver (2.6×10⁻¹⁷); Breast_Mammary_Tissue (1.1×10⁻¹⁶); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻¹⁶); Artery_Coronary (6.9×10⁻¹⁶); Esophagus_Muscularis (1.4×10⁻¹²); Adrenal_Gland (1.1×10⁻¹¹); Ovary (3.5×10⁻¹⁰); Pancreas (1.6×10⁻⁰⁹); Esophagus_Mucosa (3.1×10⁻⁰⁹); Adipose_Visceral_Omentum (6.2×10⁻⁰⁹)</t>
+          <t>Artery_Aorta (1.3×10⁻⁴⁷); Thyroid (5.7×10⁻⁴³); Artery_Tibial (2.2×10⁻⁴²); Nerve_Tibial (5×10⁻⁴²); Adipose_Subcutaneous (6.5×10⁻²⁴); Skin_Sun_Exposed_Lower_leg (8×10⁻²²); Heart_Atrial_Appendage (9.2×10⁻²²); Liver (2.6×10⁻¹⁷); Breast_Mammary_Tissue (1.1×10⁻¹⁶); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻¹⁶); Artery_Coronary (6.9×10⁻¹⁶); Esophagus_Muscularis (1.4×10⁻¹²); Adrenal_Gland (1.1×10⁻¹¹); Ovary (3.5×10⁻¹⁰); Pancreas (1.6×10⁻⁹); Esophagus_Mucosa (3.1×10⁻⁹); Adipose_Visceral_Omentum (6.2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -3696,7 +3710,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (6.4×10⁻⁷³); Artery_Tibial (7×10⁻⁷³); Artery_Aorta (3.6×10⁻⁶⁵); Nerve_Tibial (6.1×10⁻⁴¹); Lung (1.5×10⁻⁴⁰); Artery_Coronary (2.5×10⁻²⁴); Heart_Atrial_Appendage (3×10⁻²³); Testis (7.1×10⁻²²); Esophagus_Muscularis (7.6×10⁻¹⁹); Adipose_Subcutaneous (9.3×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (9.4×10⁻¹⁸); Thyroid (4.1×10⁻¹⁴); Adipose_Visceral_Omentum (2.9×10⁻¹³); Esophagus_Gastroesophageal_Junction (2.8×10⁻¹²); Stomach (1.7×10⁻¹⁰); Muscle_Skeletal (2×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (8.4×10⁻¹⁰); Brain_Cerebellum (1.8×10⁻⁰⁹); Pancreas (2.5×10⁻⁰⁹); Breast_Mammary_Tissue (1.4×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (6.4×10⁻⁷³); Artery_Tibial (7×10⁻⁷³); Artery_Aorta (3.6×10⁻⁶⁵); Nerve_Tibial (6.1×10⁻⁴¹); Lung (1.5×10⁻⁴⁰); Artery_Coronary (2.5×10⁻²⁴); Heart_Atrial_Appendage (3×10⁻²³); Testis (7.1×10⁻²²); Esophagus_Muscularis (7.6×10⁻¹⁹); Adipose_Subcutaneous (9.3×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (9.4×10⁻¹⁸); Thyroid (4.1×10⁻¹⁴); Adipose_Visceral_Omentum (2.9×10⁻¹³); Esophagus_Gastroesophageal_Junction (2.8×10⁻¹²); Stomach (1.7×10⁻¹⁰); Muscle_Skeletal (2×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (8.4×10⁻¹⁰); Brain_Cerebellum (1.8×10⁻⁹); Pancreas (2.5×10⁻⁹); Breast_Mammary_Tissue (1.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -3912,7 +3926,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Adipose_Subcutaneous (8.9×10⁻³⁰); Adipose_Visceral_Omentum (1.4×10⁻²⁰); Nerve_Tibial (2.4×10⁻⁰⁹)</t>
+          <t>Adipose_Subcutaneous (8.9×10⁻³⁰); Adipose_Visceral_Omentum (1.4×10⁻²⁰); Nerve_Tibial (2.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -4172,7 +4186,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Artery_Aorta (2.3×10⁻⁶¹); Testis (2.3×10⁻⁴⁵); Thyroid (4.3×10⁻³¹); Nerve_Tibial (6.1×10⁻²²); Adipose_Subcutaneous (8.3×10⁻²²); Brain_Cerebellum (9.8×10⁻²²); Esophagus_Muscularis (6.1×10⁻¹⁷); Brain_Cerebellar_Hemisphere (8.7×10⁻¹⁷); Minor_Salivary_Gland (1.5×10⁻¹⁶); Adipose_Visceral_Omentum (2.4×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (9.7×10⁻¹⁶); Esophagus_Mucosa (6.1×10⁻¹³); Colon_Transverse (2.8×10⁻¹²); Stomach (3.1×10⁻¹²); Heart_Left_Ventricle (1.2×10⁻¹⁰); Breast_Mammary_Tissue (2.2×10⁻¹⁰); Muscle_Skeletal (1.8×10⁻⁰⁹); Spleen (6.2×10⁻⁰⁹)</t>
+          <t>Artery_Aorta (2.3×10⁻⁶¹); Testis (2.3×10⁻⁴⁵); Thyroid (4.3×10⁻³¹); Nerve_Tibial (6.1×10⁻²²); Adipose_Subcutaneous (8.3×10⁻²²); Brain_Cerebellum (9.8×10⁻²²); Esophagus_Muscularis (6.1×10⁻¹⁷); Brain_Cerebellar_Hemisphere (8.7×10⁻¹⁷); Minor_Salivary_Gland (1.5×10⁻¹⁶); Adipose_Visceral_Omentum (2.4×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (9.7×10⁻¹⁶); Esophagus_Mucosa (6.1×10⁻¹³); Colon_Transverse (2.8×10⁻¹²); Stomach (3.1×10⁻¹²); Heart_Left_Ventricle (1.2×10⁻¹⁰); Breast_Mammary_Tissue (2.2×10⁻¹⁰); Muscle_Skeletal (1.8×10⁻⁹); Spleen (6.2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -4284,7 +4298,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Skin_Not_Sun_Exposed_Suprapubic (2.9×10⁻⁴³); Skin_Sun_Exposed_Lower_leg (1.5×10⁻²¹); Artery_Tibial (4.7×10⁻¹⁸); Pancreas (4.8×10⁻¹⁷); Esophagus_Mucosa (8×10⁻¹⁶); Artery_Aorta (4.7×10⁻⁰⁹); Brain_Cerebellum (8.3×10⁻⁰⁹); Brain_Cerebellar_Hemisphere (1×10⁻⁰⁸)</t>
+          <t>Skin_Not_Sun_Exposed_Suprapubic (2.9×10⁻⁴³); Skin_Sun_Exposed_Lower_leg (1.5×10⁻²¹); Artery_Tibial (4.7×10⁻¹⁸); Pancreas (4.8×10⁻¹⁷); Esophagus_Mucosa (8×10⁻¹⁶); Artery_Aorta (4.7×10⁻⁹); Brain_Cerebellum (8.3×10⁻⁹); Brain_Cerebellar_Hemisphere (1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -4396,7 +4410,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (5.8×10⁻¹¹⁶); Skin_Not_Sun_Exposed_Suprapubic (8.5×10⁻⁷⁸); Cells_Cultured_fibroblasts (2.7×10⁻⁶⁷); Adipose_Subcutaneous (1.9×10⁻⁶²); Brain_Cerebellum (1.9×10⁻³⁵); Colon_Sigmoid (2.9×10⁻³²); Brain_Cerebellar_Hemisphere (8×10⁻³²); Lung (1.4×10⁻²⁹); Adrenal_Gland (4×10⁻²⁸); Muscle_Skeletal (1×10⁻²⁵); Breast_Mammary_Tissue (1.5×10⁻²⁴); Artery_Tibial (3.5×10⁻²³); Esophagus_Mucosa (7×10⁻²³); Brain_Cortex (4.4×10⁻²¹); Brain_Caudate_basal_ganglia (5.8×10⁻²⁰); Colon_Transverse (3.9×10⁻¹⁸); Testis (2.8×10⁻¹⁵); Esophagus_Muscularis (3.3×10⁻¹⁵); Brain_Nucleus_accumbens_basal_ganglia (4.3×10⁻¹⁵); Esophagus_Gastroesophageal_Junction (1.9×10⁻¹²); Brain_Putamen_basal_ganglia (3.9×10⁻¹¹); Pancreas (6.7×10⁻¹¹); Brain_Frontal_Cortex_BA9 (7.4×10⁻¹¹); Brain_Anterior_cingulate_cortex_BA24 (9.4×10⁻¹¹); Stomach (1.1×10⁻¹⁰); Adipose_Visceral_Omentum (7.4×10⁻¹⁰); Spleen (8.5×10⁻⁰⁹)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (5.8×10⁻¹¹⁶); Skin_Not_Sun_Exposed_Suprapubic (8.5×10⁻⁷⁸); Cells_Cultured_fibroblasts (2.7×10⁻⁶⁷); Adipose_Subcutaneous (1.9×10⁻⁶²); Brain_Cerebellum (1.9×10⁻³⁵); Colon_Sigmoid (2.9×10⁻³²); Brain_Cerebellar_Hemisphere (8×10⁻³²); Lung (1.4×10⁻²⁹); Adrenal_Gland (4×10⁻²⁸); Muscle_Skeletal (1×10⁻²⁵); Breast_Mammary_Tissue (1.5×10⁻²⁴); Artery_Tibial (3.5×10⁻²³); Esophagus_Mucosa (7×10⁻²³); Brain_Cortex (4.4×10⁻²¹); Brain_Caudate_basal_ganglia (5.8×10⁻²⁰); Colon_Transverse (3.9×10⁻¹⁸); Testis (2.8×10⁻¹⁵); Esophagus_Muscularis (3.3×10⁻¹⁵); Brain_Nucleus_accumbens_basal_ganglia (4.3×10⁻¹⁵); Esophagus_Gastroesophageal_Junction (1.9×10⁻¹²); Brain_Putamen_basal_ganglia (3.9×10⁻¹¹); Pancreas (6.7×10⁻¹¹); Brain_Frontal_Cortex_BA9 (7.4×10⁻¹¹); Brain_Anterior_cingulate_cortex_BA24 (9.4×10⁻¹¹); Stomach (1.1×10⁻¹⁰); Adipose_Visceral_Omentum (7.4×10⁻¹⁰); Spleen (8.5×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -4656,7 +4670,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Lung (3.2×10⁻⁰⁹); Artery_Aorta (7.8×10⁻⁰⁹)</t>
+          <t>Lung (3.2×10⁻⁹); Artery_Aorta (7.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -5028,7 +5042,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1×10⁻¹⁷); Skin_Not_Sun_Exposed_Suprapubic (9.7×10⁻¹⁵); Esophagus_Mucosa (2.3×10⁻⁰⁸); Prostate (2.4×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1×10⁻¹⁷); Skin_Not_Sun_Exposed_Suprapubic (9.7×10⁻¹⁵); Esophagus_Mucosa (2.3×10⁻⁸); Prostate (2.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr"/>
@@ -5156,7 +5170,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -5556,7 +5570,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (4.6×10⁻⁵⁸); Skin_Not_Sun_Exposed_Suprapubic (2.3×10⁻³⁵); Heart_Left_Ventricle (1.1×10⁻³⁰); Adipose_Subcutaneous (4.9×10⁻²⁹); Nerve_Tibial (8.4×10⁻¹⁶); Heart_Atrial_Appendage (1.1×10⁻¹¹); Artery_Tibial (8×10⁻¹¹); Esophagus_Gastroesophageal_Junction (6.9×10⁻⁰⁹); Esophagus_Muscularis (1.1×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (4.6×10⁻⁵⁸); Skin_Not_Sun_Exposed_Suprapubic (2.3×10⁻³⁵); Heart_Left_Ventricle (1.1×10⁻³⁰); Adipose_Subcutaneous (4.9×10⁻²⁹); Nerve_Tibial (8.4×10⁻¹⁶); Heart_Atrial_Appendage (1.1×10⁻¹¹); Artery_Tibial (8×10⁻¹¹); Esophagus_Gastroesophageal_Junction (6.9×10⁻⁹); Esophagus_Muscularis (1.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -5688,7 +5702,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Testis (3.5×10⁻⁵⁴); Lung (3.1×10⁻⁵²); Esophagus_Muscularis (1.3×10⁻³⁰); Esophagus_Gastroesophageal_Junction (1×10⁻²⁶); Adrenal_Gland (5.7×10⁻²⁴); Brain_Caudate_basal_ganglia (5.3×10⁻²²); Brain_Nucleus_accumbens_basal_ganglia (1.1×10⁻²⁰); Spleen (1.2×10⁻²⁰); Heart_Atrial_Appendage (1.7×10⁻²⁰); Brain_Putamen_basal_ganglia (2.5×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (1.8×10⁻¹²); Esophagus_Mucosa (2.6×10⁻¹²); Adipose_Subcutaneous (1.8×10⁻¹⁰); Pancreas (2.6×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (1.8×10⁻⁰⁹); Pituitary (5.6×10⁻⁰⁹); Brain_Cerebellum (6.4×10⁻⁰⁹); Nerve_Tibial (2×10⁻⁰⁸)</t>
+          <t>Testis (3.5×10⁻⁵⁴); Lung (3.1×10⁻⁵²); Esophagus_Muscularis (1.3×10⁻³⁰); Esophagus_Gastroesophageal_Junction (1×10⁻²⁶); Adrenal_Gland (5.7×10⁻²⁴); Brain_Caudate_basal_ganglia (5.3×10⁻²²); Brain_Nucleus_accumbens_basal_ganglia (1.1×10⁻²⁰); Spleen (1.2×10⁻²⁰); Heart_Atrial_Appendage (1.7×10⁻²⁰); Brain_Putamen_basal_ganglia (2.5×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (1.8×10⁻¹²); Esophagus_Mucosa (2.6×10⁻¹²); Adipose_Subcutaneous (1.8×10⁻¹⁰); Pancreas (2.6×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (1.8×10⁻⁹); Pituitary (5.6×10⁻⁹); Brain_Cerebellum (6.4×10⁻⁹); Nerve_Tibial (2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -6200,7 +6214,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Testis (8.4×10⁻¹⁰); Adrenal_Gland (1.7×10⁻⁰⁹)</t>
+          <t>Testis (8.4×10⁻¹⁰); Adrenal_Gland (1.7×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -6312,7 +6326,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Thyroid (1.5×10⁻²⁵); Skin_Sun_Exposed_Lower_leg (4.9×10⁻¹²); Artery_Coronary (3.6×10⁻⁰⁸); Vagina (5×10⁻⁰⁸)</t>
+          <t>Thyroid (1.5×10⁻²⁵); Skin_Sun_Exposed_Lower_leg (4.9×10⁻¹²); Artery_Coronary (3.6×10⁻⁸); Vagina (5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -6532,7 +6546,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (3.5×10⁻¹¹); Brain_Cerebellar_Hemisphere (1.3×10⁻⁰⁹); Thyroid (2.5×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (3.5×10⁻¹¹); Brain_Cerebellar_Hemisphere (1.3×10⁻⁹); Thyroid (2.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr"/>
@@ -6904,7 +6918,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Brain_Cerebellar_Hemisphere (9.6×10⁻²¹); Brain_Cerebellum (1.3×10⁻¹⁹); Brain_Cortex (1.7×10⁻¹⁴); Nerve_Tibial (9.1×10⁻¹¹); Testis (1.3×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (6.6×10⁻¹⁰); Brain_Caudate_basal_ganglia (4×10⁻⁰⁹); Brain_Putamen_basal_ganglia (7.1×10⁻⁰⁹); Heart_Atrial_Appendage (2.6×10⁻⁰⁸); Brain_Anterior_cingulate_cortex_BA24 (4.6×10⁻⁰⁸)</t>
+          <t>Brain_Cerebellar_Hemisphere (9.6×10⁻²¹); Brain_Cerebellum (1.3×10⁻¹⁹); Brain_Cortex (1.7×10⁻¹⁴); Nerve_Tibial (9.1×10⁻¹¹); Testis (1.3×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (6.6×10⁻¹⁰); Brain_Caudate_basal_ganglia (4×10⁻⁹); Brain_Putamen_basal_ganglia (7.1×10⁻⁹); Heart_Atrial_Appendage (2.6×10⁻⁸); Brain_Anterior_cingulate_cortex_BA24 (4.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -7012,7 +7026,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Artery_Tibial (2.7×10⁻⁴⁹); Artery_Aorta (4.5×10⁻²⁶); Artery_Coronary (6.4×10⁻¹⁴); Heart_Left_Ventricle (1.2×10⁻⁰⁹); Colon_Transverse (3×10⁻⁰⁸); Heart_Atrial_Appendage (4×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (2.7×10⁻⁴⁹); Artery_Aorta (4.5×10⁻²⁶); Artery_Coronary (6.4×10⁻¹⁴); Heart_Left_Ventricle (1.2×10⁻⁹); Colon_Transverse (3×10⁻⁸); Heart_Atrial_Appendage (4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -7904,7 +7918,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Spleen (1.6×10⁻¹¹); Adipose_Visceral_Omentum (3.8×10⁻⁰⁸)</t>
+          <t>Spleen (1.6×10⁻¹¹); Adipose_Visceral_Omentum (3.8×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -8044,7 +8058,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Lung (8×10⁻⁵⁷); Heart_Left_Ventricle (1×10⁻³²); Cells_Cultured_fibroblasts (2.3×10⁻²⁴); Testis (1.5×10⁻⁰⁹)</t>
+          <t>Lung (8×10⁻⁵⁷); Heart_Left_Ventricle (1×10⁻³²); Cells_Cultured_fibroblasts (2.3×10⁻²⁴); Testis (1.5×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -8260,7 +8274,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (2.6×10⁻³²); Liver (1.7×10⁻²⁹); Brain_Cerebellum (2.9×10⁻²⁶); Brain_Cerebellar_Hemisphere (7.6×10⁻²¹); Brain_Nucleus_accumbens_basal_ganglia (4.8×10⁻¹²); Brain_Frontal_Cortex_BA9 (4.7×10⁻¹⁰); Brain_Spinal_cord_cervical_c-1 (8.9×10⁻¹⁰); Spleen (1.8×10⁻⁰⁹); Brain_Putamen_basal_ganglia (2.4×10⁻⁰⁹); Testis (1.1×10⁻⁰⁸); Brain_Caudate_basal_ganglia (2.8×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (2.6×10⁻³²); Liver (1.7×10⁻²⁹); Brain_Cerebellum (2.9×10⁻²⁶); Brain_Cerebellar_Hemisphere (7.6×10⁻²¹); Brain_Nucleus_accumbens_basal_ganglia (4.8×10⁻¹²); Brain_Frontal_Cortex_BA9 (4.7×10⁻¹⁰); Brain_Spinal_cord_cervical_c-1 (8.9×10⁻¹⁰); Spleen (1.8×10⁻⁹); Brain_Putamen_basal_ganglia (2.4×10⁻⁹); Testis (1.1×10⁻⁸); Brain_Caudate_basal_ganglia (2.8×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -8368,7 +8382,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Pancreas (4.4×10⁻¹⁷); Thyroid (2×10⁻¹⁵); Nerve_Tibial (4.1×10⁻¹²); Lung (7.9×10⁻¹²); Artery_Aorta (4.3×10⁻¹¹); Adipose_Subcutaneous (1.6×10⁻⁰⁹); Brain_Hippocampus (4.9×10⁻⁰⁹); Colon_Sigmoid (5.4×10⁻⁰⁹)</t>
+          <t>Pancreas (4.4×10⁻¹⁷); Thyroid (2×10⁻¹⁵); Nerve_Tibial (4.1×10⁻¹²); Lung (7.9×10⁻¹²); Artery_Aorta (4.3×10⁻¹¹); Adipose_Subcutaneous (1.6×10⁻⁹); Brain_Hippocampus (4.9×10⁻⁹); Colon_Sigmoid (5.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -8872,7 +8886,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>Adipose_Subcutaneous (1.6×10⁻⁸³); Adipose_Visceral_Omentum (8.9×10⁻⁶⁴); Breast_Mammary_Tissue (1.1×10⁻³¹); Thyroid (3.6×10⁻¹⁶); Esophagus_Mucosa (1.3×10⁻¹⁴); Skin_Sun_Exposed_Lower_leg (1×10⁻¹¹); Nerve_Tibial (1.7×10⁻⁰⁹); Minor_Salivary_Gland (3.6×10⁻⁰⁸)</t>
+          <t>Adipose_Subcutaneous (1.6×10⁻⁸³); Adipose_Visceral_Omentum (8.9×10⁻⁶⁴); Breast_Mammary_Tissue (1.1×10⁻³¹); Thyroid (3.6×10⁻¹⁶); Esophagus_Mucosa (1.3×10⁻¹⁴); Skin_Sun_Exposed_Lower_leg (1×10⁻¹¹); Nerve_Tibial (1.7×10⁻⁹); Minor_Salivary_Gland (3.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -9216,7 +9230,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Adrenal_Gland (3.6×10⁻⁰⁹)</t>
+          <t>Adrenal_Gland (3.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -9504,7 +9518,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Artery_Aorta (6.6×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (9.3×10⁻¹⁸); Skin_Not_Sun_Exposed_Suprapubic (8.2×10⁻¹⁵); Adipose_Subcutaneous (1×10⁻¹⁰); Nerve_Tibial (1.4×10⁻¹⁰); Esophagus_Mucosa (2×10⁻⁰⁹)</t>
+          <t>Artery_Aorta (6.6×10⁻¹⁹); Skin_Sun_Exposed_Lower_leg (9.3×10⁻¹⁸); Skin_Not_Sun_Exposed_Suprapubic (8.2×10⁻¹⁵); Adipose_Subcutaneous (1×10⁻¹⁰); Nerve_Tibial (1.4×10⁻¹⁰); Esophagus_Mucosa (2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -9744,7 +9758,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (1.4×10⁻¹³); Adipose_Subcutaneous (7.6×10⁻¹⁰); Skin_Sun_Exposed_Lower_leg (9.8×10⁻¹⁰); Pancreas (1.8×10⁻⁰⁹); Brain_Cerebellum (4.6×10⁻⁰⁹); Brain_Cortex (4.6×10⁻⁰⁹); Skin_Not_Sun_Exposed_Suprapubic (1.4×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (1.4×10⁻¹³); Adipose_Subcutaneous (7.6×10⁻¹⁰); Skin_Sun_Exposed_Lower_leg (9.8×10⁻¹⁰); Pancreas (1.8×10⁻⁹); Brain_Cerebellum (4.6×10⁻⁹); Brain_Cortex (4.6×10⁻⁹); Skin_Not_Sun_Exposed_Suprapubic (1.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr"/>
@@ -9888,7 +9902,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Lung (1.8×10⁻⁶⁷); Cells_Cultured_fibroblasts (5.9×10⁻⁵²); Muscle_Skeletal (2.3×10⁻²⁶); Adipose_Subcutaneous (2×10⁻¹⁹); Esophagus_Mucosa (2.1×10⁻¹⁵); Adipose_Visceral_Omentum (3×10⁻¹⁵); Skin_Sun_Exposed_Lower_leg (1.9×10⁻¹²); Artery_Tibial (3.3×10⁻¹²); Esophagus_Muscularis (4.7×10⁻¹²); Heart_Left_Ventricle (1.4×10⁻¹¹); Heart_Atrial_Appendage (6.7×10⁻¹⁰); Esophagus_Gastroesophageal_Junction (1.6×10⁻⁰⁹); Thyroid (8.4×10⁻⁰⁹)</t>
+          <t>Lung (1.8×10⁻⁶⁷); Cells_Cultured_fibroblasts (5.9×10⁻⁵²); Muscle_Skeletal (2.3×10⁻²⁶); Adipose_Subcutaneous (2×10⁻¹⁹); Esophagus_Mucosa (2.1×10⁻¹⁵); Adipose_Visceral_Omentum (3×10⁻¹⁵); Skin_Sun_Exposed_Lower_leg (1.9×10⁻¹²); Artery_Tibial (3.3×10⁻¹²); Esophagus_Muscularis (4.7×10⁻¹²); Heart_Left_Ventricle (1.4×10⁻¹¹); Heart_Atrial_Appendage (6.7×10⁻¹⁰); Esophagus_Gastroesophageal_Junction (1.6×10⁻⁹); Thyroid (8.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -10032,7 +10046,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1.3×10⁻¹⁸); Brain_Cortex (4.2×10⁻¹⁴); Brain_Nucleus_accumbens_basal_ganglia (1.3×10⁻¹¹); Brain_Caudate_basal_ganglia (1.7×10⁻¹¹); Pancreas (1.3×10⁻¹⁰); Brain_Cerebellum (1.3×10⁻⁰⁹); Muscle_Skeletal (1.5×10⁻⁰⁹); Brain_Frontal_Cortex_BA9 (1.6×10⁻⁰⁹); Skin_Sun_Exposed_Lower_leg (2×10⁻⁰⁸); Cells_Cultured_fibroblasts (4.6×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (1.3×10⁻¹⁸); Brain_Cortex (4.2×10⁻¹⁴); Brain_Nucleus_accumbens_basal_ganglia (1.3×10⁻¹¹); Brain_Caudate_basal_ganglia (1.7×10⁻¹¹); Pancreas (1.3×10⁻¹⁰); Brain_Cerebellum (1.3×10⁻⁹); Muscle_Skeletal (1.5×10⁻⁹); Brain_Frontal_Cortex_BA9 (1.6×10⁻⁹); Skin_Sun_Exposed_Lower_leg (2×10⁻⁸); Cells_Cultured_fibroblasts (4.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -10140,7 +10154,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Brain_Cerebellar_Hemisphere (2.5×10⁻¹⁰); Prostate (1.4×10⁻⁰⁸); Colon_Transverse (4.3×10⁻⁰⁸)</t>
+          <t>Brain_Cerebellar_Hemisphere (2.5×10⁻¹⁰); Prostate (1.4×10⁻⁸); Colon_Transverse (4.3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -10272,7 +10286,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Brain_Nucleus_accumbens_basal_ganglia (3.8×10⁻¹⁴); Brain_Putamen_basal_ganglia (8.1×10⁻¹⁴); Brain_Caudate_basal_ganglia (4.2×10⁻¹³); Artery_Tibial (1.8×10⁻¹²); Lung (2.4×10⁻¹²); Esophagus_Muscularis (1.8×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (8×10⁻¹⁰); Nerve_Tibial (1.3×10⁻⁰⁹); Colon_Transverse (1.9×10⁻⁰⁹); Esophagus_Gastroesophageal_Junction (2.1×10⁻⁰⁸)</t>
+          <t>Brain_Nucleus_accumbens_basal_ganglia (3.8×10⁻¹⁴); Brain_Putamen_basal_ganglia (8.1×10⁻¹⁴); Brain_Caudate_basal_ganglia (4.2×10⁻¹³); Artery_Tibial (1.8×10⁻¹²); Lung (2.4×10⁻¹²); Esophagus_Muscularis (1.8×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (8×10⁻¹⁰); Nerve_Tibial (1.3×10⁻⁹); Colon_Transverse (1.9×10⁻⁹); Esophagus_Gastroesophageal_Junction (2.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -10420,7 +10434,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Artery_Tibial (3.3×10⁻¹⁵); Brain_Cerebellum (2×10⁻¹²); Testis (1.1×10⁻⁰⁹)</t>
+          <t>Artery_Tibial (3.3×10⁻¹⁵); Brain_Cerebellum (2×10⁻¹²); Testis (1.1×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -10564,7 +10578,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1×10⁻⁰⁹); Skin_Not_Sun_Exposed_Suprapubic (2.1×10⁻⁰⁸); Skin_Sun_Exposed_Lower_leg (2.7×10⁻⁰⁸); Artery_Aorta (3.6×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (1×10⁻⁹); Skin_Not_Sun_Exposed_Suprapubic (2.1×10⁻⁸); Skin_Sun_Exposed_Lower_leg (2.7×10⁻⁸); Artery_Aorta (3.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -10688,7 +10702,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (2.7×10⁻³³); Adipose_Subcutaneous (3.4×10⁻²³); Breast_Mammary_Tissue (4.1×10⁻¹⁶); Artery_Tibial (6.4×10⁻¹⁴); Adipose_Visceral_Omentum (3.5×10⁻¹³); Brain_Putamen_basal_ganglia (4.6×10⁻⁰⁹); Skin_Sun_Exposed_Lower_leg (5.4×10⁻⁰⁹); Esophagus_Mucosa (1.2×10⁻⁰⁸); Brain_Nucleus_accumbens_basal_ganglia (1.2×10⁻⁰⁸); Minor_Salivary_Gland (2.4×10⁻⁰⁸); Artery_Aorta (3×10⁻⁰⁸); Esophagus_Muscularis (3.7×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (2.7×10⁻³³); Adipose_Subcutaneous (3.4×10⁻²³); Breast_Mammary_Tissue (4.1×10⁻¹⁶); Artery_Tibial (6.4×10⁻¹⁴); Adipose_Visceral_Omentum (3.5×10⁻¹³); Brain_Putamen_basal_ganglia (4.6×10⁻⁹); Skin_Sun_Exposed_Lower_leg (5.4×10⁻⁹); Esophagus_Mucosa (1.2×10⁻⁸); Brain_Nucleus_accumbens_basal_ganglia (1.2×10⁻⁸); Minor_Salivary_Gland (2.4×10⁻⁸); Artery_Aorta (3×10⁻⁸); Esophagus_Muscularis (3.7×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -10948,7 +10962,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (2.9×10⁻⁷⁸); Brain_Nucleus_accumbens_basal_ganglia (4.4×10⁻³²); Brain_Caudate_basal_ganglia (1.1×10⁻²⁶); Brain_Hypothalamus (8.3×10⁻²³); Brain_Putamen_basal_ganglia (3.4×10⁻²⁰); Brain_Hippocampus (5.3×10⁻¹⁹); Brain_Cortex (7.8×10⁻¹⁹); Esophagus_Muscularis (1.3×10⁻¹⁸); Brain_Frontal_Cortex_BA9 (3.5×10⁻¹⁸); Testis (4.9×10⁻¹⁷); Brain_Anterior_cingulate_cortex_BA24 (8.5×10⁻¹⁶); Muscle_Skeletal (5.8×10⁻¹⁵); Brain_Substantia_nigra (1.9×10⁻¹⁴); Esophagus_Gastroesophageal_Junction (6.5×10⁻¹⁴); Brain_Amygdala (2.3×10⁻¹³); Brain_Spinal_cord_cervical_c-1 (4.6×10⁻⁰⁹); Brain_Cerebellar_Hemisphere (4.1×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (2.9×10⁻⁷⁸); Brain_Nucleus_accumbens_basal_ganglia (4.4×10⁻³²); Brain_Caudate_basal_ganglia (1.1×10⁻²⁶); Brain_Hypothalamus (8.3×10⁻²³); Brain_Putamen_basal_ganglia (3.4×10⁻²⁰); Brain_Hippocampus (5.3×10⁻¹⁹); Brain_Cortex (7.8×10⁻¹⁹); Esophagus_Muscularis (1.3×10⁻¹⁸); Brain_Frontal_Cortex_BA9 (3.5×10⁻¹⁸); Testis (4.9×10⁻¹⁷); Brain_Anterior_cingulate_cortex_BA24 (8.5×10⁻¹⁶); Muscle_Skeletal (5.8×10⁻¹⁵); Brain_Substantia_nigra (1.9×10⁻¹⁴); Esophagus_Gastroesophageal_Junction (6.5×10⁻¹⁴); Brain_Amygdala (2.3×10⁻¹³); Brain_Spinal_cord_cervical_c-1 (4.6×10⁻⁹); Brain_Cerebellar_Hemisphere (4.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr"/>
@@ -11088,7 +11102,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Spleen (1.9×10⁻²³); Heart_Left_Ventricle (5.2×10⁻⁰⁹)</t>
+          <t>Spleen (1.9×10⁻²³); Heart_Left_Ventricle (5.2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -11220,7 +11234,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (1.1×10⁻¹⁷); Artery_Tibial (7.5×10⁻¹³); Muscle_Skeletal (4.4×10⁻¹¹); Adipose_Subcutaneous (1.3×10⁻¹⁰); Nerve_Tibial (1.3×10⁻⁰⁹); Thyroid (3×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (1.1×10⁻¹⁷); Artery_Tibial (7.5×10⁻¹³); Muscle_Skeletal (4.4×10⁻¹¹); Adipose_Subcutaneous (1.3×10⁻¹⁰); Nerve_Tibial (1.3×10⁻⁹); Thyroid (3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -11364,7 +11378,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Thyroid (1.9×10⁻⁵⁹); Pituitary (2.6×10⁻⁴¹); Lung (1.4×10⁻³⁹); Nerve_Tibial (1.6×10⁻³⁵); Spleen (3.3×10⁻²³); Colon_Sigmoid (9.6×10⁻²³); Prostate (1.4×10⁻¹⁶); Testis (2.3×10⁻¹⁵); Uterus (4.3×10⁻¹⁵); Ovary (1.8×10⁻¹⁴); Cells_EBV-transformed_lymphocytes (4.6×10⁻¹⁴); Brain_Caudate_basal_ganglia (9.7×10⁻¹⁴); Brain_Hippocampus (1.1×10⁻¹³); Brain_Spinal_cord_cervical_c-1 (3.9×10⁻¹³); Adrenal_Gland (4.3×10⁻¹³); Brain_Nucleus_accumbens_basal_ganglia (1.8×10⁻¹²); Esophagus_Gastroesophageal_Junction (7.9×10⁻¹²); Brain_Hypothalamus (9.3×10⁻¹²); Esophagus_Muscularis (1.3×10⁻¹¹); Breast_Mammary_Tissue (1.7×10⁻¹¹); Small_Intestine_Terminal_Ileum (4×10⁻¹¹); Brain_Cortex (1.3×10⁻¹⁰); Brain_Putamen_basal_ganglia (2.2×10⁻¹⁰); Colon_Transverse (2.9×10⁻⁰⁸)</t>
+          <t>Thyroid (1.9×10⁻⁵⁹); Pituitary (2.6×10⁻⁴¹); Lung (1.4×10⁻³⁹); Nerve_Tibial (1.6×10⁻³⁵); Spleen (3.3×10⁻²³); Colon_Sigmoid (9.6×10⁻²³); Prostate (1.4×10⁻¹⁶); Testis (2.3×10⁻¹⁵); Uterus (4.3×10⁻¹⁵); Ovary (1.8×10⁻¹⁴); Cells_EBV-transformed_lymphocytes (4.6×10⁻¹⁴); Brain_Caudate_basal_ganglia (9.7×10⁻¹⁴); Brain_Hippocampus (1.1×10⁻¹³); Brain_Spinal_cord_cervical_c-1 (3.9×10⁻¹³); Adrenal_Gland (4.3×10⁻¹³); Brain_Nucleus_accumbens_basal_ganglia (1.8×10⁻¹²); Esophagus_Gastroesophageal_Junction (7.9×10⁻¹²); Brain_Hypothalamus (9.3×10⁻¹²); Esophagus_Muscularis (1.3×10⁻¹¹); Breast_Mammary_Tissue (1.7×10⁻¹¹); Small_Intestine_Terminal_Ileum (4×10⁻¹¹); Brain_Cortex (1.3×10⁻¹⁰); Brain_Putamen_basal_ganglia (2.2×10⁻¹⁰); Colon_Transverse (2.9×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -11596,7 +11610,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Stomach (4.9×10⁻⁰⁹)</t>
+          <t>Stomach (4.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -11824,7 +11838,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Adipose_Subcutaneous (2.7×10⁻²⁹); Esophagus_Muscularis (4.9×10⁻²⁹); Artery_Tibial (5.2×10⁻²⁷); Nerve_Tibial (4.8×10⁻²⁵); Esophagus_Gastroesophageal_Junction (9×10⁻²¹); Thyroid (1.9×10⁻¹⁸); Heart_Left_Ventricle (8.3×10⁻¹⁸); Adipose_Visceral_Omentum (1.5×10⁻¹⁷); Lung (2.4×10⁻¹⁶); Colon_Sigmoid (7.4×10⁻¹⁵); Muscle_Skeletal (5.6×10⁻¹⁴); Artery_Aorta (1.2×10⁻¹³); Heart_Atrial_Appendage (2.2×10⁻¹³); Esophagus_Mucosa (5.8×10⁻¹³); Stomach (4.6×10⁻¹¹); Adrenal_Gland (5.5×10⁻¹¹); Artery_Coronary (5.2×10⁻¹⁰); Spleen (1.3×10⁻⁰⁸)</t>
+          <t>Adipose_Subcutaneous (2.7×10⁻²⁹); Esophagus_Muscularis (4.9×10⁻²⁹); Artery_Tibial (5.2×10⁻²⁷); Nerve_Tibial (4.8×10⁻²⁵); Esophagus_Gastroesophageal_Junction (9×10⁻²¹); Thyroid (1.9×10⁻¹⁸); Heart_Left_Ventricle (8.3×10⁻¹⁸); Adipose_Visceral_Omentum (1.5×10⁻¹⁷); Lung (2.4×10⁻¹⁶); Colon_Sigmoid (7.4×10⁻¹⁵); Muscle_Skeletal (5.6×10⁻¹⁴); Artery_Aorta (1.2×10⁻¹³); Heart_Atrial_Appendage (2.2×10⁻¹³); Esophagus_Mucosa (5.8×10⁻¹³); Stomach (4.6×10⁻¹¹); Adrenal_Gland (5.5×10⁻¹¹); Artery_Coronary (5.2×10⁻¹⁰); Spleen (1.3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -12208,7 +12222,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>Pancreas (6.1×10⁻²²); Cells_Cultured_fibroblasts (7.1×10⁻¹⁰); Thyroid (3.4×10⁻⁰⁹); Artery_Aorta (3.5×10⁻⁰⁹); Esophagus_Muscularis (6×10⁻⁰⁹); Lung (1.2×10⁻⁰⁸); Artery_Tibial (2.5×10⁻⁰⁸)</t>
+          <t>Pancreas (6.1×10⁻²²); Cells_Cultured_fibroblasts (7.1×10⁻¹⁰); Thyroid (3.4×10⁻⁹); Artery_Aorta (3.5×10⁻⁹); Esophagus_Muscularis (6×10⁻⁹); Lung (1.2×10⁻⁸); Artery_Tibial (2.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -12352,7 +12366,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Heart_Atrial_Appendage (1.1×10⁻⁰⁸)</t>
+          <t>Heart_Atrial_Appendage (1.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -12576,7 +12590,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Muscle_Skeletal (1×10⁻⁴²); Thyroid (1.1×10⁻⁴¹); Esophagus_Mucosa (2×10⁻³⁹); Skin_Sun_Exposed_Lower_leg (3.7×10⁻²⁷); Esophagus_Muscularis (2.5×10⁻²⁶); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻²²); Lung (2.8×10⁻²⁰); Artery_Aorta (1×10⁻¹⁸); Nerve_Tibial (3.1×10⁻¹⁸); Artery_Tibial (1.3×10⁻¹⁷); Pancreas (1.6×10⁻¹⁷); Cells_Cultured_fibroblasts (4.2×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (2×10⁻¹⁵); Adipose_Subcutaneous (1.4×10⁻¹⁴); Testis (2.4×10⁻¹⁴); Stomach (6×10⁻¹⁴); Adrenal_Gland (9.1×10⁻¹³); Prostate (1.1×10⁻¹²); Colon_Sigmoid (2.1×10⁻¹¹); Liver (1.9×10⁻¹⁰); Colon_Transverse (2.9×10⁻¹⁰); Minor_Salivary_Gland (3.4×10⁻¹⁰); Heart_Left_Ventricle (7.4×10⁻¹⁰); Adipose_Visceral_Omentum (3.7×10⁻⁰⁹); Heart_Atrial_Appendage (4.7×10⁻⁰⁹); Small_Intestine_Terminal_Ileum (1.1×10⁻⁰⁸); Spleen (1.9×10⁻⁰⁸)</t>
+          <t>Muscle_Skeletal (1×10⁻⁴²); Thyroid (1.1×10⁻⁴¹); Esophagus_Mucosa (2×10⁻³⁹); Skin_Sun_Exposed_Lower_leg (3.7×10⁻²⁷); Esophagus_Muscularis (2.5×10⁻²⁶); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻²²); Lung (2.8×10⁻²⁰); Artery_Aorta (1×10⁻¹⁸); Nerve_Tibial (3.1×10⁻¹⁸); Artery_Tibial (1.3×10⁻¹⁷); Pancreas (1.6×10⁻¹⁷); Cells_Cultured_fibroblasts (4.2×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (2×10⁻¹⁵); Adipose_Subcutaneous (1.4×10⁻¹⁴); Testis (2.4×10⁻¹⁴); Stomach (6×10⁻¹⁴); Adrenal_Gland (9.1×10⁻¹³); Prostate (1.1×10⁻¹²); Colon_Sigmoid (2.1×10⁻¹¹); Liver (1.9×10⁻¹⁰); Colon_Transverse (2.9×10⁻¹⁰); Minor_Salivary_Gland (3.4×10⁻¹⁰); Heart_Left_Ventricle (7.4×10⁻¹⁰); Adipose_Visceral_Omentum (3.7×10⁻⁹); Heart_Atrial_Appendage (4.7×10⁻⁹); Small_Intestine_Terminal_Ileum (1.1×10⁻⁸); Spleen (1.9×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -12936,7 +12950,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Prostate (1.4×10⁻¹⁰); Adipose_Subcutaneous (7.5×10⁻¹⁰); Artery_Tibial (6.9×10⁻⁰⁹); Testis (1.6×10⁻⁰⁸)</t>
+          <t>Prostate (1.4×10⁻¹⁰); Adipose_Subcutaneous (7.5×10⁻¹⁰); Artery_Tibial (6.9×10⁻⁹); Testis (1.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -13728,7 +13742,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>Esophagus_Muscularis (1.9×10⁻⁹⁷); Esophagus_Gastroesophageal_Junction (1×10⁻⁴⁵); Thyroid (4.8×10⁻³²); Artery_Aorta (4.8×10⁻²⁹); Heart_Atrial_Appendage (8.9×10⁻²⁴); Heart_Left_Ventricle (2.3×10⁻¹⁵); Adipose_Subcutaneous (5×10⁻¹⁴); Artery_Tibial (3.3×10⁻¹³); Breast_Mammary_Tissue (1.3×10⁻¹¹); Nerve_Tibial (6.2×10⁻¹⁰); Artery_Coronary (6.4×10⁻¹⁰); Esophagus_Mucosa (3.6×10⁻⁰⁹); Adipose_Visceral_Omentum (1.2×10⁻⁰⁸); Lung (2.4×10⁻⁰⁸)</t>
+          <t>Esophagus_Muscularis (1.9×10⁻⁹⁷); Esophagus_Gastroesophageal_Junction (1×10⁻⁴⁵); Thyroid (4.8×10⁻³²); Artery_Aorta (4.8×10⁻²⁹); Heart_Atrial_Appendage (8.9×10⁻²⁴); Heart_Left_Ventricle (2.3×10⁻¹⁵); Adipose_Subcutaneous (5×10⁻¹⁴); Artery_Tibial (3.3×10⁻¹³); Breast_Mammary_Tissue (1.3×10⁻¹¹); Nerve_Tibial (6.2×10⁻¹⁰); Artery_Coronary (6.4×10⁻¹⁰); Esophagus_Mucosa (3.6×10⁻⁹); Adipose_Visceral_Omentum (1.2×10⁻⁸); Lung (2.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -13976,7 +13990,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (2.1×10⁻³⁹); Brain_Cerebellar_Hemisphere (3.3×10⁻³⁹); Esophagus_Mucosa (3.6×10⁻³⁷); Skin_Sun_Exposed_Lower_leg (7.1×10⁻²²); Heart_Atrial_Appendage (1.4×10⁻²¹); Skin_Not_Sun_Exposed_Suprapubic (2×10⁻²¹); Lung (5.8×10⁻¹⁸); Esophagus_Muscularis (8×10⁻¹⁷); Esophagus_Gastroesophageal_Junction (1.5×10⁻⁰⁸)</t>
+          <t>Brain_Cerebellum (2.1×10⁻³⁹); Brain_Cerebellar_Hemisphere (3.3×10⁻³⁹); Esophagus_Mucosa (3.6×10⁻³⁷); Skin_Sun_Exposed_Lower_leg (7.1×10⁻²²); Heart_Atrial_Appendage (1.4×10⁻²¹); Skin_Not_Sun_Exposed_Suprapubic (2×10⁻²¹); Lung (5.8×10⁻¹⁸); Esophagus_Muscularis (8×10⁻¹⁷); Esophagus_Gastroesophageal_Junction (1.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -14476,7 +14490,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>Skin_Not_Sun_Exposed_Suprapubic (2.4×10⁻¹⁶); Skin_Sun_Exposed_Lower_leg (8.8×10⁻¹³); Artery_Tibial (1.5×10⁻⁰⁹); Spleen (7.2×10⁻⁰⁹); Heart_Atrial_Appendage (3.7×10⁻⁰⁸)</t>
+          <t>Skin_Not_Sun_Exposed_Suprapubic (2.4×10⁻¹⁶); Skin_Sun_Exposed_Lower_leg (8.8×10⁻¹³); Artery_Tibial (1.5×10⁻⁹); Spleen (7.2×10⁻⁹); Heart_Atrial_Appendage (3.7×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -14584,7 +14598,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (3.1×10⁻²⁷); Brain_Cerebellar_Hemisphere (1.5×10⁻¹⁹); Brain_Cortex (6.4×10⁻¹⁵); Artery_Tibial (1.2×10⁻¹⁰); Artery_Aorta (3.6×10⁻¹⁰); Heart_Atrial_Appendage (3.6×10⁻¹⁰); Pancreas (4.3×10⁻⁰⁸)</t>
+          <t>Brain_Cerebellum (3.1×10⁻²⁷); Brain_Cerebellar_Hemisphere (1.5×10⁻¹⁹); Brain_Cortex (6.4×10⁻¹⁵); Artery_Tibial (1.2×10⁻¹⁰); Artery_Aorta (3.6×10⁻¹⁰); Heart_Atrial_Appendage (3.6×10⁻¹⁰); Pancreas (4.3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
@@ -14692,7 +14706,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>Pancreas (8.9×10⁻²³); Thyroid (3.5×10⁻²⁰); Pituitary (2.7×10⁻¹⁴); Ovary (1.2×10⁻¹⁰); Heart_Atrial_Appendage (1.4×10⁻⁰⁹)</t>
+          <t>Pancreas (8.9×10⁻²³); Thyroid (3.5×10⁻²⁰); Pituitary (2.7×10⁻¹⁴); Ovary (1.2×10⁻¹⁰); Heart_Atrial_Appendage (1.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -14800,7 +14814,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (5.8×10⁻¹⁰⁸); Esophagus_Muscularis (1.6×10⁻⁰⁹)</t>
+          <t>Cells_Cultured_fibroblasts (5.8×10⁻¹⁰⁸); Esophagus_Muscularis (1.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr"/>
@@ -15072,7 +15086,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (1.8×10⁻³⁴); Muscle_Skeletal (2.7×10⁻²⁶); Skin_Sun_Exposed_Lower_leg (1.5×10⁻¹⁵); Esophagus_Mucosa (1.5×10⁻¹⁴); Esophagus_Muscularis (1.1×10⁻¹³); Skin_Not_Sun_Exposed_Suprapubic (4.8×10⁻¹²); Vagina (1.9×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (1.8×10⁻³⁴); Muscle_Skeletal (2.7×10⁻²⁶); Skin_Sun_Exposed_Lower_leg (1.5×10⁻¹⁵); Esophagus_Mucosa (1.5×10⁻¹⁴); Esophagus_Muscularis (1.1×10⁻¹³); Skin_Not_Sun_Exposed_Suprapubic (4.8×10⁻¹²); Vagina (1.9×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -15188,7 +15202,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (1.1×10⁻⁸¹); Esophagus_Muscularis (2.6×10⁻⁴⁴); Thyroid (2.5×10⁻³⁸); Esophagus_Gastroesophageal_Junction (1.6×10⁻²⁶); Esophagus_Mucosa (1.3×10⁻²²); Adipose_Visceral_Omentum (6.9×10⁻²²); Artery_Aorta (6×10⁻¹⁹); Adipose_Subcutaneous (2.2×10⁻¹⁷); Skin_Sun_Exposed_Lower_leg (2.1×10⁻¹⁴); Colon_Sigmoid (4×10⁻¹¹); Prostate (3.4×10⁻¹⁰); Breast_Mammary_Tissue (4.3×10⁻¹⁰); Colon_Transverse (1.5×10⁻⁰⁸); Skin_Not_Sun_Exposed_Suprapubic (5×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (1.1×10⁻⁸¹); Esophagus_Muscularis (2.6×10⁻⁴⁴); Thyroid (2.5×10⁻³⁸); Esophagus_Gastroesophageal_Junction (1.6×10⁻²⁶); Esophagus_Mucosa (1.3×10⁻²²); Adipose_Visceral_Omentum (6.9×10⁻²²); Artery_Aorta (6×10⁻¹⁹); Adipose_Subcutaneous (2.2×10⁻¹⁷); Skin_Sun_Exposed_Lower_leg (2.1×10⁻¹⁴); Colon_Sigmoid (4×10⁻¹¹); Prostate (3.4×10⁻¹⁰); Breast_Mammary_Tissue (4.3×10⁻¹⁰); Colon_Transverse (1.5×10⁻⁸); Skin_Not_Sun_Exposed_Suprapubic (5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -15300,7 +15314,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>Esophagus_Mucosa (7.4×10⁻²⁹); Thyroid (3×10⁻¹⁵); Liver (7.4×10⁻⁰⁹)</t>
+          <t>Esophagus_Mucosa (7.4×10⁻²⁹); Thyroid (3×10⁻¹⁵); Liver (7.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -15420,7 +15434,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1.4×10⁻³⁴); Skin_Not_Sun_Exposed_Suprapubic (1.1×10⁻²⁷); Cells_Cultured_fibroblasts (1.9×10⁻²⁰); Esophagus_Mucosa (3.3×10⁻¹⁵); Adrenal_Gland (4.6×10⁻⁰⁹); Artery_Aorta (1.2×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1.4×10⁻³⁴); Skin_Not_Sun_Exposed_Suprapubic (1.1×10⁻²⁷); Cells_Cultured_fibroblasts (1.9×10⁻²⁰); Esophagus_Mucosa (3.3×10⁻¹⁵); Adrenal_Gland (4.6×10⁻⁹); Artery_Aorta (1.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -15528,7 +15542,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (5.5×10⁻¹⁶); Muscle_Skeletal (4.2×10⁻¹⁵); Artery_Aorta (1.2×10⁻¹⁴); Artery_Tibial (4.2×10⁻¹⁴); Brain_Caudate_basal_ganglia (7×10⁻¹¹); Colon_Sigmoid (2.9×10⁻⁰⁹); Lung (9.2×10⁻⁰⁹); Brain_Frontal_Cortex_BA9 (1×10⁻⁰⁸); Esophagus_Muscularis (2.3×10⁻⁰⁸); Thyroid (2.4×10⁻⁰⁸); Brain_Anterior_cingulate_cortex_BA24 (3.4×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (5.5×10⁻¹⁶); Muscle_Skeletal (4.2×10⁻¹⁵); Artery_Aorta (1.2×10⁻¹⁴); Artery_Tibial (4.2×10⁻¹⁴); Brain_Caudate_basal_ganglia (7×10⁻¹¹); Colon_Sigmoid (2.9×10⁻⁹); Lung (9.2×10⁻⁹); Brain_Frontal_Cortex_BA9 (1×10⁻⁸); Esophagus_Muscularis (2.3×10⁻⁸); Thyroid (2.4×10⁻⁸); Brain_Anterior_cingulate_cortex_BA24 (3.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -15780,7 +15794,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>Esophagus_Gastroesophageal_Junction (2.1×10⁻¹²); Esophagus_Muscularis (4.9×10⁻¹²); Artery_Tibial (6.6×10⁻¹²); Artery_Aorta (1.4×10⁻¹⁰); Lung (3.1×10⁻¹⁰); Thyroid (7.1×10⁻¹⁰); Adipose_Subcutaneous (3.6×10⁻⁰⁹); Pancreas (9.4×10⁻⁰⁹)</t>
+          <t>Esophagus_Gastroesophageal_Junction (2.1×10⁻¹²); Esophagus_Muscularis (4.9×10⁻¹²); Artery_Tibial (6.6×10⁻¹²); Artery_Aorta (1.4×10⁻¹⁰); Lung (3.1×10⁻¹⁰); Thyroid (7.1×10⁻¹⁰); Adipose_Subcutaneous (3.6×10⁻⁹); Pancreas (9.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -16396,7 +16410,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1.6×10⁻⁷⁵); Skin_Not_Sun_Exposed_Suprapubic (1×10⁻⁴²); Testis (6×10⁻²¹); Brain_Cortex (3.8×10⁻⁰⁹)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1.6×10⁻⁷⁵); Skin_Not_Sun_Exposed_Suprapubic (1×10⁻⁴²); Testis (6×10⁻²¹); Brain_Cortex (3.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -16540,7 +16554,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1.9×10⁻⁸²); Skin_Not_Sun_Exposed_Suprapubic (4.3×10⁻⁵⁶); Muscle_Skeletal (8.6×10⁻³³); Pancreas (3.9×10⁻¹³); Brain_Hippocampus (9.6×10⁻¹³); Nerve_Tibial (2.5×10⁻¹¹); Brain_Cortex (8.6×10⁻¹¹); Esophagus_Mucosa (3.2×10⁻¹⁰); Vagina (8×10⁻¹⁰); Thyroid (1.5×10⁻⁰⁹); Brain_Spinal_cord_cervical_c-1 (7.6×10⁻⁰⁹); Brain_Frontal_Cortex_BA9 (3.1×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1.9×10⁻⁸²); Skin_Not_Sun_Exposed_Suprapubic (4.3×10⁻⁵⁶); Muscle_Skeletal (8.6×10⁻³³); Pancreas (3.9×10⁻¹³); Brain_Hippocampus (9.6×10⁻¹³); Nerve_Tibial (2.5×10⁻¹¹); Brain_Cortex (8.6×10⁻¹¹); Esophagus_Mucosa (3.2×10⁻¹⁰); Vagina (8×10⁻¹⁰); Thyroid (1.5×10⁻⁹); Brain_Spinal_cord_cervical_c-1 (7.6×10⁻⁹); Brain_Frontal_Cortex_BA9 (3.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -16780,7 +16794,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>Thyroid (6×10⁻³⁹); Nerve_Tibial (3×10⁻³⁸); Artery_Tibial (5.8×10⁻³⁸); Adrenal_Gland (5.9×10⁻²⁶); Liver (2.2×10⁻²²); Pancreas (6.5×10⁻¹³); Heart_Left_Ventricle (7.7×10⁻¹³); Muscle_Skeletal (1.7×10⁻¹²); Adipose_Subcutaneous (6.8×10⁻¹²); Spleen (1×10⁻¹¹); Adipose_Visceral_Omentum (1.4×10⁻¹¹); Artery_Coronary (4.3×10⁻⁰⁹); Skin_Sun_Exposed_Lower_leg (7.7×10⁻⁰⁹)</t>
+          <t>Thyroid (6×10⁻³⁹); Nerve_Tibial (3×10⁻³⁸); Artery_Tibial (5.8×10⁻³⁸); Adrenal_Gland (5.9×10⁻²⁶); Liver (2.2×10⁻²²); Pancreas (6.5×10⁻¹³); Heart_Left_Ventricle (7.7×10⁻¹³); Muscle_Skeletal (1.7×10⁻¹²); Adipose_Subcutaneous (6.8×10⁻¹²); Spleen (1×10⁻¹¹); Adipose_Visceral_Omentum (1.4×10⁻¹¹); Artery_Coronary (4.3×10⁻⁹); Skin_Sun_Exposed_Lower_leg (7.7×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -16888,7 +16902,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (7.9×10⁻⁴⁵); Testis (1.4×10⁻¹⁷); Lung (1×10⁻¹⁶); Adrenal_Gland (1.8×10⁻⁰⁹)</t>
+          <t>Nerve_Tibial (7.9×10⁻⁴⁵); Testis (1.4×10⁻¹⁷); Lung (1×10⁻¹⁶); Adrenal_Gland (1.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -17112,7 +17126,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>Testis (3.7×10⁻⁵⁵); Brain_Cerebellum (2.7×10⁻⁵²); Brain_Cortex (5.3×10⁻⁴¹); Pituitary (5.7×10⁻³⁹); Brain_Cerebellar_Hemisphere (7.3×10⁻³⁸); Brain_Frontal_Cortex_BA9 (3.5×10⁻³²); Brain_Nucleus_accumbens_basal_ganglia (2×10⁻²⁹); Brain_Hypothalamus (1.4×10⁻²⁸); Brain_Caudate_basal_ganglia (8.7×10⁻²⁶); Brain_Anterior_cingulate_cortex_BA24 (1.5×10⁻²¹); Prostate (4.2×10⁻¹⁸); Lung (1.7×10⁻¹⁵); Brain_Hippocampus (2.1×10⁻¹⁵); Brain_Amygdala (1.2×10⁻¹³); Brain_Putamen_basal_ganglia (3.7×10⁻¹³); Thyroid (1×10⁻¹¹); Esophagus_Mucosa (5.3×10⁻¹¹); Brain_Substantia_nigra (2.9×10⁻¹⁰); Adrenal_Gland (1.6×10⁻⁰⁹); Muscle_Skeletal (2.8×10⁻⁰⁸)</t>
+          <t>Testis (3.7×10⁻⁵⁵); Brain_Cerebellum (2.7×10⁻⁵²); Brain_Cortex (5.3×10⁻⁴¹); Pituitary (5.7×10⁻³⁹); Brain_Cerebellar_Hemisphere (7.3×10⁻³⁸); Brain_Frontal_Cortex_BA9 (3.5×10⁻³²); Brain_Nucleus_accumbens_basal_ganglia (2×10⁻²⁹); Brain_Hypothalamus (1.4×10⁻²⁸); Brain_Caudate_basal_ganglia (8.7×10⁻²⁶); Brain_Anterior_cingulate_cortex_BA24 (1.5×10⁻²¹); Prostate (4.2×10⁻¹⁸); Lung (1.7×10⁻¹⁵); Brain_Hippocampus (2.1×10⁻¹⁵); Brain_Amygdala (1.2×10⁻¹³); Brain_Putamen_basal_ganglia (3.7×10⁻¹³); Thyroid (1×10⁻¹¹); Esophagus_Mucosa (5.3×10⁻¹¹); Brain_Substantia_nigra (2.9×10⁻¹⁰); Adrenal_Gland (1.6×10⁻⁹); Muscle_Skeletal (2.8×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr">
@@ -17488,7 +17502,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>Heart_Atrial_Appendage (1.5×10⁻²¹); Esophagus_Muscularis (3.2×10⁻²¹); Adrenal_Gland (1.7×10⁻¹²); Heart_Left_Ventricle (9.1×10⁻¹¹); Liver (1×10⁻¹⁰); Colon_Transverse (1.7×10⁻⁰⁸)</t>
+          <t>Heart_Atrial_Appendage (1.5×10⁻²¹); Esophagus_Muscularis (3.2×10⁻²¹); Adrenal_Gland (1.7×10⁻¹²); Heart_Left_Ventricle (9.1×10⁻¹¹); Liver (1×10⁻¹⁰); Colon_Transverse (1.7×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -17864,7 +17878,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>Esophagus_Mucosa (7.8×10⁻⁷³); Testis (1.1×10⁻⁴⁹); Colon_Transverse (5.4×10⁻¹⁸); Muscle_Skeletal (1.2×10⁻¹⁶); Artery_Tibial (8.1×10⁻¹⁴); Stomach (1.3×10⁻¹³); Adipose_Subcutaneous (1.1×10⁻¹¹); Small_Intestine_Terminal_Ileum (2.3×10⁻¹¹); Colon_Sigmoid (9.2×10⁻¹⁰); Esophagus_Muscularis (3×10⁻⁰⁹); Heart_Atrial_Appendage (7.6×10⁻⁰⁹); Heart_Left_Ventricle (1.2×10⁻⁰⁸); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻⁰⁸); Cells_Cultured_fibroblasts (1.5×10⁻⁰⁸); Brain_Nucleus_accumbens_basal_ganglia (1.5×10⁻⁰⁸); Brain_Cortex (2.1×10⁻⁰⁸)</t>
+          <t>Esophagus_Mucosa (7.8×10⁻⁷³); Testis (1.1×10⁻⁴⁹); Colon_Transverse (5.4×10⁻¹⁸); Muscle_Skeletal (1.2×10⁻¹⁶); Artery_Tibial (8.1×10⁻¹⁴); Stomach (1.3×10⁻¹³); Adipose_Subcutaneous (1.1×10⁻¹¹); Small_Intestine_Terminal_Ileum (2.3×10⁻¹¹); Colon_Sigmoid (9.2×10⁻¹⁰); Esophagus_Muscularis (3×10⁻⁹); Heart_Atrial_Appendage (7.6×10⁻⁹); Heart_Left_Ventricle (1.2×10⁻⁸); Skin_Not_Sun_Exposed_Suprapubic (1.3×10⁻⁸); Cells_Cultured_fibroblasts (1.5×10⁻⁸); Brain_Nucleus_accumbens_basal_ganglia (1.5×10⁻⁸); Brain_Cortex (2.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
@@ -17976,7 +17990,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (2.8×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (2.8×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr"/>
@@ -18120,7 +18134,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1.4×10⁻¹⁴); Cells_Cultured_fibroblasts (8.1×10⁻¹³); Cells_EBV-transformed_lymphocytes (9.5×10⁻⁰⁹)</t>
+          <t>Artery_Tibial (1.4×10⁻¹⁴); Cells_Cultured_fibroblasts (8.1×10⁻¹³); Cells_EBV-transformed_lymphocytes (9.5×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -18264,7 +18278,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>Artery_Tibial (3.4×10⁻⁵⁶); Cells_Cultured_fibroblasts (1.4×10⁻²⁸); Artery_Aorta (6.2×10⁻¹⁰); Adipose_Subcutaneous (1.1×10⁻⁰⁹); Nerve_Tibial (5.9×10⁻⁰⁹); Prostate (1×10⁻⁰⁸); Adrenal_Gland (2.4×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (3.4×10⁻⁵⁶); Cells_Cultured_fibroblasts (1.4×10⁻²⁸); Artery_Aorta (6.2×10⁻¹⁰); Adipose_Subcutaneous (1.1×10⁻⁹); Nerve_Tibial (5.9×10⁻⁹); Prostate (1×10⁻⁸); Adrenal_Gland (2.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -18516,7 +18530,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>Adrenal_Gland (1.2×10⁻³⁵); Pituitary (3×10⁻³⁵); Liver (1.3×10⁻³¹); Ovary (3.9×10⁻²⁶); Pancreas (2.9×10⁻²⁵); Testis (5.6×10⁻¹⁸); Prostate (7.4×10⁻¹⁸); Nerve_Tibial (3.1×10⁻¹³); Lung (3.6×10⁻¹³); Adipose_Visceral_Omentum (2×10⁻¹¹); Breast_Mammary_Tissue (2.6×10⁻¹⁰); Small_Intestine_Terminal_Ileum (9.1×10⁻¹⁰); Brain_Hypothalamus (2.3×10⁻⁰⁹); Colon_Transverse (1.2×10⁻⁰⁸); Heart_Atrial_Appendage (4.4×10⁻⁰⁸)</t>
+          <t>Adrenal_Gland (1.2×10⁻³⁵); Pituitary (3×10⁻³⁵); Liver (1.3×10⁻³¹); Ovary (3.9×10⁻²⁶); Pancreas (2.9×10⁻²⁵); Testis (5.6×10⁻¹⁸); Prostate (7.4×10⁻¹⁸); Nerve_Tibial (3.1×10⁻¹³); Lung (3.6×10⁻¹³); Adipose_Visceral_Omentum (2×10⁻¹¹); Breast_Mammary_Tissue (2.6×10⁻¹⁰); Small_Intestine_Terminal_Ileum (9.1×10⁻¹⁰); Brain_Hypothalamus (2.3×10⁻⁹); Colon_Transverse (1.2×10⁻⁸); Heart_Atrial_Appendage (4.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -18636,7 +18650,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (3.2×10⁻¹³); Artery_Aorta (3.6×10⁻¹¹); Colon_Sigmoid (2.6×10⁻⁰⁹)</t>
+          <t>Cells_Cultured_fibroblasts (3.2×10⁻¹³); Artery_Aorta (3.6×10⁻¹¹); Colon_Sigmoid (2.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -18780,7 +18794,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (5.9×10⁻⁹¹); Esophagus_Mucosa (3.3×10⁻⁵³); Heart_Atrial_Appendage (3.9×10⁻⁵²); Artery_Tibial (3.2×10⁻¹⁷); Heart_Left_Ventricle (2.6×10⁻¹³); Thyroid (3.6×10⁻¹³); Cells_Cultured_fibroblasts (3×10⁻¹²); Skin_Sun_Exposed_Lower_leg (1.1×10⁻⁰⁹); Minor_Salivary_Gland (1.1×10⁻⁰⁹)</t>
+          <t>Nerve_Tibial (5.9×10⁻⁹¹); Esophagus_Mucosa (3.3×10⁻⁵³); Heart_Atrial_Appendage (3.9×10⁻⁵²); Artery_Tibial (3.2×10⁻¹⁷); Heart_Left_Ventricle (2.6×10⁻¹³); Thyroid (3.6×10⁻¹³); Cells_Cultured_fibroblasts (3×10⁻¹²); Skin_Sun_Exposed_Lower_leg (1.1×10⁻⁹); Minor_Salivary_Gland (1.1×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
@@ -18924,7 +18938,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (5.1×10⁻¹⁵); Ovary (5.3×10⁻¹⁵); Muscle_Skeletal (2.1×10⁻¹²); Brain_Caudate_basal_ganglia (1.4×10⁻¹¹); Nerve_Tibial (3.3×10⁻¹⁰); Adipose_Subcutaneous (5.1×10⁻¹⁰); Lung (6.5×10⁻¹⁰); Adipose_Visceral_Omentum (7.4×10⁻¹⁰); Testis (3.3×10⁻⁰⁹); Breast_Mammary_Tissue (4.5×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (5.1×10⁻¹⁵); Ovary (5.3×10⁻¹⁵); Muscle_Skeletal (2.1×10⁻¹²); Brain_Caudate_basal_ganglia (1.4×10⁻¹¹); Nerve_Tibial (3.3×10⁻¹⁰); Adipose_Subcutaneous (5.1×10⁻¹⁰); Lung (6.5×10⁻¹⁰); Adipose_Visceral_Omentum (7.4×10⁻¹⁰); Testis (3.3×10⁻⁹); Breast_Mammary_Tissue (4.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -19056,7 +19070,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (4.3×10⁻²⁴); Ovary (1.5×10⁻¹²); Skin_Not_Sun_Exposed_Suprapubic (1.4×10⁻¹¹); Testis (5.9×10⁻¹¹); Brain_Cortex (1.6×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (4.3×10⁻²⁴); Ovary (1.5×10⁻¹²); Skin_Not_Sun_Exposed_Suprapubic (1.4×10⁻¹¹); Testis (5.9×10⁻¹¹); Brain_Cortex (1.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -19196,7 +19210,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>Colon_Transverse (4.1×10⁻¹²); Cells_Cultured_fibroblasts (3.9×10⁻⁰⁹)</t>
+          <t>Colon_Transverse (4.1×10⁻¹²); Cells_Cultured_fibroblasts (3.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -19312,7 +19326,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>Testis (6.5×10⁻²⁵); Brain_Cerebellar_Hemisphere (4.6×10⁻²³); Brain_Cerebellum (5.7×10⁻²²); Brain_Putamen_basal_ganglia (4×10⁻¹⁶); Brain_Caudate_basal_ganglia (8.4×10⁻¹⁶); Pituitary (1.6×10⁻¹¹); Brain_Cortex (2.5×10⁻¹⁰); Brain_Hippocampus (1.4×10⁻⁰⁸); Brain_Nucleus_accumbens_basal_ganglia (1.6×10⁻⁰⁸)</t>
+          <t>Testis (6.5×10⁻²⁵); Brain_Cerebellar_Hemisphere (4.6×10⁻²³); Brain_Cerebellum (5.7×10⁻²²); Brain_Putamen_basal_ganglia (4×10⁻¹⁶); Brain_Caudate_basal_ganglia (8.4×10⁻¹⁶); Pituitary (1.6×10⁻¹¹); Brain_Cortex (2.5×10⁻¹⁰); Brain_Hippocampus (1.4×10⁻⁸); Brain_Nucleus_accumbens_basal_ganglia (1.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr"/>
@@ -19452,7 +19466,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>Adipose_Subcutaneous (4.6×10⁻²⁰); Spleen (7.7×10⁻¹⁹); Skin_Not_Sun_Exposed_Suprapubic (2.6×10⁻¹⁷); Skin_Sun_Exposed_Lower_leg (5.8×10⁻¹⁶); Testis (9.1×10⁻¹⁴); Adipose_Visceral_Omentum (1.3×10⁻¹²); Breast_Mammary_Tissue (1.7×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (1.3×10⁻¹⁰); Brain_Hypothalamus (3.1×10⁻¹⁰); Pituitary (5.1×10⁻¹⁰); Esophagus_Mucosa (2.6×10⁻⁰⁹); Nerve_Tibial (3.5×10⁻⁰⁹); Thyroid (6.4×10⁻⁰⁹); Adrenal_Gland (1.9×10⁻⁰⁸)</t>
+          <t>Adipose_Subcutaneous (4.6×10⁻²⁰); Spleen (7.7×10⁻¹⁹); Skin_Not_Sun_Exposed_Suprapubic (2.6×10⁻¹⁷); Skin_Sun_Exposed_Lower_leg (5.8×10⁻¹⁶); Testis (9.1×10⁻¹⁴); Adipose_Visceral_Omentum (1.3×10⁻¹²); Breast_Mammary_Tissue (1.7×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (1.3×10⁻¹⁰); Brain_Hypothalamus (3.1×10⁻¹⁰); Pituitary (5.1×10⁻¹⁰); Esophagus_Mucosa (2.6×10⁻⁹); Nerve_Tibial (3.5×10⁻⁹); Thyroid (6.4×10⁻⁹); Adrenal_Gland (1.9×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -19560,7 +19574,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>Adipose_Visceral_Omentum (2×10⁻¹⁶); Cells_Cultured_fibroblasts (3.6×10⁻¹³); Artery_Aorta (4.8×10⁻¹²); Uterus (7×10⁻¹⁰); Artery_Coronary (9.3×10⁻⁰⁹); Brain_Cerebellum (1.1×10⁻⁰⁸); Artery_Tibial (1.4×10⁻⁰⁸)</t>
+          <t>Adipose_Visceral_Omentum (2×10⁻¹⁶); Cells_Cultured_fibroblasts (3.6×10⁻¹³); Artery_Aorta (4.8×10⁻¹²); Uterus (7×10⁻¹⁰); Artery_Coronary (9.3×10⁻⁹); Brain_Cerebellum (1.1×10⁻⁸); Artery_Tibial (1.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -19812,7 +19826,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1.9×10⁻⁰⁹)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -20076,7 +20090,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>Testis (2.3×10⁻²³); Lung (1×10⁻²⁰); Adipose_Visceral_Omentum (5.4×10⁻¹⁶); Esophagus_Muscularis (3.3×10⁻¹⁴); Adipose_Subcutaneous (3.3×10⁻¹⁰); Colon_Transverse (9.1×10⁻¹⁰); Adrenal_Gland (5.8×10⁻⁰⁹); Spleen (7.1×10⁻⁰⁹)</t>
+          <t>Testis (2.3×10⁻²³); Lung (1×10⁻²⁰); Adipose_Visceral_Omentum (5.4×10⁻¹⁶); Esophagus_Muscularis (3.3×10⁻¹⁴); Adipose_Subcutaneous (3.3×10⁻¹⁰); Colon_Transverse (9.1×10⁻¹⁰); Adrenal_Gland (5.8×10⁻⁹); Spleen (7.1×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -20188,7 +20202,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>Skin_Not_Sun_Exposed_Suprapubic (7.9×10⁻⁷¹); Skin_Sun_Exposed_Lower_leg (2.9×10⁻⁶⁶); Testis (9.6×10⁻²³); Adrenal_Gland (6.2×10⁻¹⁸); Esophagus_Muscularis (5.5×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (3.5×10⁻⁰⁸)</t>
+          <t>Skin_Not_Sun_Exposed_Suprapubic (7.9×10⁻⁷¹); Skin_Sun_Exposed_Lower_leg (2.9×10⁻⁶⁶); Testis (9.6×10⁻²³); Adrenal_Gland (6.2×10⁻¹⁸); Esophagus_Muscularis (5.5×10⁻¹⁶); Esophagus_Gastroesophageal_Junction (3.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -20300,7 +20314,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (6.2×10⁻²⁷); Skin_Not_Sun_Exposed_Suprapubic (6.3×10⁻²⁷); Esophagus_Mucosa (7.1×10⁻²¹); Artery_Aorta (2.1×10⁻¹⁵); Esophagus_Muscularis (3.3×10⁻¹²); Heart_Atrial_Appendage (1.4×10⁻⁰⁹)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (6.2×10⁻²⁷); Skin_Not_Sun_Exposed_Suprapubic (6.3×10⁻²⁷); Esophagus_Mucosa (7.1×10⁻²¹); Artery_Aorta (2.1×10⁻¹⁵); Esophagus_Muscularis (3.3×10⁻¹²); Heart_Atrial_Appendage (1.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -20408,7 +20422,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1.6×10⁻³⁷); Nerve_Tibial (3.5×10⁻²⁴); Artery_Aorta (9×10⁻¹⁸); Esophagus_Mucosa (1.2×10⁻¹⁷); Lung (6×10⁻¹⁵); Breast_Mammary_Tissue (2.2×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (1.9×10⁻⁰⁹); Colon_Sigmoid (6×10⁻⁰⁹); Esophagus_Gastroesophageal_Junction (2.4×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (1.6×10⁻³⁷); Nerve_Tibial (3.5×10⁻²⁴); Artery_Aorta (9×10⁻¹⁸); Esophagus_Mucosa (1.2×10⁻¹⁷); Lung (6×10⁻¹⁵); Breast_Mammary_Tissue (2.2×10⁻¹⁰); Skin_Not_Sun_Exposed_Suprapubic (1.9×10⁻⁹); Colon_Sigmoid (6×10⁻⁹); Esophagus_Gastroesophageal_Junction (2.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -20516,7 +20530,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>Muscle_Skeletal (6.2×10⁻³⁰); Thyroid (1.6×10⁻²⁷); Adrenal_Gland (2.8×10⁻²²); Heart_Left_Ventricle (1.5×10⁻¹⁹); Adipose_Subcutaneous (6.6×10⁻¹⁶); Adipose_Visceral_Omentum (6×10⁻¹⁵); Lung (8.7×10⁻¹⁵); Liver (3.2×10⁻¹²); Breast_Mammary_Tissue (5.4×10⁻¹¹); Nerve_Tibial (5.9×10⁻⁰⁹)</t>
+          <t>Muscle_Skeletal (6.2×10⁻³⁰); Thyroid (1.6×10⁻²⁷); Adrenal_Gland (2.8×10⁻²²); Heart_Left_Ventricle (1.5×10⁻¹⁹); Adipose_Subcutaneous (6.6×10⁻¹⁶); Adipose_Visceral_Omentum (6×10⁻¹⁵); Lung (8.7×10⁻¹⁵); Liver (3.2×10⁻¹²); Breast_Mammary_Tissue (5.4×10⁻¹¹); Nerve_Tibial (5.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr">
@@ -20760,7 +20774,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>Artery_Tibial (2.5×10⁻⁴³); Artery_Aorta (2.4×10⁻¹²); Brain_Hypothalamus (6.6×10⁻¹⁰); Adipose_Visceral_Omentum (1.1×10⁻⁰⁹); Adipose_Subcutaneous (2.8×10⁻⁰⁹)</t>
+          <t>Artery_Tibial (2.5×10⁻⁴³); Artery_Aorta (2.4×10⁻¹²); Brain_Hypothalamus (6.6×10⁻¹⁰); Adipose_Visceral_Omentum (1.1×10⁻⁹); Adipose_Subcutaneous (2.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
@@ -20908,7 +20922,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>Adipose_Subcutaneous (2.6×10⁻²¹); Adipose_Visceral_Omentum (5.6×10⁻¹⁵); Esophagus_Muscularis (2.3×10⁻¹³); Nerve_Tibial (2.4×10⁻⁰⁹); Esophagus_Gastroesophageal_Junction (3.9×10⁻⁰⁹); Skin_Sun_Exposed_Lower_leg (4×10⁻⁰⁹); Breast_Mammary_Tissue (7.4×10⁻⁰⁹); Colon_Transverse (3.3×10⁻⁰⁸); Heart_Left_Ventricle (4.4×10⁻⁰⁸)</t>
+          <t>Adipose_Subcutaneous (2.6×10⁻²¹); Adipose_Visceral_Omentum (5.6×10⁻¹⁵); Esophagus_Muscularis (2.3×10⁻¹³); Nerve_Tibial (2.4×10⁻⁹); Esophagus_Gastroesophageal_Junction (3.9×10⁻⁹); Skin_Sun_Exposed_Lower_leg (4×10⁻⁹); Breast_Mammary_Tissue (7.4×10⁻⁹); Colon_Transverse (3.3×10⁻⁸); Heart_Left_Ventricle (4.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
@@ -21016,7 +21030,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>Heart_Atrial_Appendage (6.5×10⁻⁰⁹); Colon_Transverse (2.6×10⁻⁰⁸); Pancreas (2.9×10⁻⁰⁸)</t>
+          <t>Heart_Atrial_Appendage (6.5×10⁻⁹); Colon_Transverse (2.6×10⁻⁸); Pancreas (2.9×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
@@ -21160,7 +21174,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>Artery_Tibial (6.9×10⁻⁷⁴); Nerve_Tibial (2.2×10⁻⁶⁶); Muscle_Skeletal (7.6×10⁻⁶¹); Adipose_Subcutaneous (5.5×10⁻⁵⁶); Thyroid (1.6×10⁻⁵⁵); Esophagus_Muscularis (1.3×10⁻⁵³); Skin_Sun_Exposed_Lower_leg (4×10⁻⁵³); Skin_Not_Sun_Exposed_Suprapubic (3×10⁻⁴⁹); Esophagus_Gastroesophageal_Junction (1.4×10⁻⁴⁵); Adipose_Visceral_Omentum (1.4×10⁻⁴³); Lung (7.7×10⁻⁴¹); Colon_Transverse (7×10⁻³⁹); Artery_Aorta (6.2×10⁻³⁴); Cells_Cultured_fibroblasts (2.1×10⁻³³); Esophagus_Mucosa (4.6×10⁻³²); Breast_Mammary_Tissue (2.5×10⁻³¹); Colon_Sigmoid (2.1×10⁻³⁰); Adrenal_Gland (6.8×10⁻²⁶); Spleen (2.3×10⁻²¹); Pituitary (2×10⁻¹⁹); Prostate (1.9×10⁻¹⁸); Artery_Coronary (4.5×10⁻¹⁸); Stomach (6.7×10⁻¹⁷); Brain_Cerebellum (2.3×10⁻¹⁶); Brain_Amygdala (2.6×10⁻¹⁵); Pancreas (2.7×10⁻¹⁵); Ovary (6.4×10⁻¹⁵); Uterus (1.2×10⁻¹⁴); Brain_Spinal_cord_cervical_c-1 (3.9×10⁻¹⁴); Brain_Hypothalamus (1.1×10⁻¹²); Brain_Cortex (2.4×10⁻¹²); Small_Intestine_Terminal_Ileum (3.4×10⁻¹²); Brain_Hippocampus (8.8×10⁻¹²); Brain_Caudate_basal_ganglia (3.9×10⁻¹¹); Brain_Putamen_basal_ganglia (5.3×10⁻¹¹); Brain_Anterior_cingulate_cortex_BA24 (7.9×10⁻¹¹); Brain_Nucleus_accumbens_basal_ganglia (1.1×10⁻¹⁰); Testis (2.5×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (3.7×10⁻¹⁰); Vagina (7.1×10⁻¹⁰); Brain_Substantia_nigra (7.7×10⁻¹⁰); Brain_Cerebellar_Hemisphere (1.2×10⁻⁰⁹); Minor_Salivary_Gland (1.9×10⁻⁰⁹); Heart_Left_Ventricle (4.6×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (6.9×10⁻⁷⁴); Nerve_Tibial (2.2×10⁻⁶⁶); Muscle_Skeletal (7.6×10⁻⁶¹); Adipose_Subcutaneous (5.5×10⁻⁵⁶); Thyroid (1.6×10⁻⁵⁵); Esophagus_Muscularis (1.3×10⁻⁵³); Skin_Sun_Exposed_Lower_leg (4×10⁻⁵³); Skin_Not_Sun_Exposed_Suprapubic (3×10⁻⁴⁹); Esophagus_Gastroesophageal_Junction (1.4×10⁻⁴⁵); Adipose_Visceral_Omentum (1.4×10⁻⁴³); Lung (7.7×10⁻⁴¹); Colon_Transverse (7×10⁻³⁹); Artery_Aorta (6.2×10⁻³⁴); Cells_Cultured_fibroblasts (2.1×10⁻³³); Esophagus_Mucosa (4.6×10⁻³²); Breast_Mammary_Tissue (2.5×10⁻³¹); Colon_Sigmoid (2.1×10⁻³⁰); Adrenal_Gland (6.8×10⁻²⁶); Spleen (2.3×10⁻²¹); Pituitary (2×10⁻¹⁹); Prostate (1.9×10⁻¹⁸); Artery_Coronary (4.5×10⁻¹⁸); Stomach (6.7×10⁻¹⁷); Brain_Cerebellum (2.3×10⁻¹⁶); Brain_Amygdala (2.6×10⁻¹⁵); Pancreas (2.7×10⁻¹⁵); Ovary (6.4×10⁻¹⁵); Uterus (1.2×10⁻¹⁴); Brain_Spinal_cord_cervical_c-1 (3.9×10⁻¹⁴); Brain_Hypothalamus (1.1×10⁻¹²); Brain_Cortex (2.4×10⁻¹²); Small_Intestine_Terminal_Ileum (3.4×10⁻¹²); Brain_Hippocampus (8.8×10⁻¹²); Brain_Caudate_basal_ganglia (3.9×10⁻¹¹); Brain_Putamen_basal_ganglia (5.3×10⁻¹¹); Brain_Anterior_cingulate_cortex_BA24 (7.9×10⁻¹¹); Brain_Nucleus_accumbens_basal_ganglia (1.1×10⁻¹⁰); Testis (2.5×10⁻¹⁰); Brain_Frontal_Cortex_BA9 (3.7×10⁻¹⁰); Vagina (7.1×10⁻¹⁰); Brain_Substantia_nigra (7.7×10⁻¹⁰); Brain_Cerebellar_Hemisphere (1.2×10⁻⁹); Minor_Salivary_Gland (1.9×10⁻⁹); Heart_Left_Ventricle (4.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
@@ -21380,7 +21394,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>Lung (6.7×10⁻⁵¹); Thyroid (2×10⁻¹⁷); Nerve_Tibial (6.7×10⁻¹⁴); Cells_Cultured_fibroblasts (2.2×10⁻¹⁰); Heart_Left_Ventricle (4.3×10⁻⁰⁸)</t>
+          <t>Lung (6.7×10⁻⁵¹); Thyroid (2×10⁻¹⁷); Nerve_Tibial (6.7×10⁻¹⁴); Cells_Cultured_fibroblasts (2.2×10⁻¹⁰); Heart_Left_Ventricle (4.3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr">
@@ -21524,7 +21538,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>Thyroid (4×10⁻⁷⁷); Heart_Atrial_Appendage (4.5×10⁻³²); Heart_Left_Ventricle (1.1×10⁻²¹); Pancreas (1.1×10⁻¹⁴); Testis (4×10⁻¹³); Artery_Aorta (4.7×10⁻⁰⁸)</t>
+          <t>Thyroid (4×10⁻⁷⁷); Heart_Atrial_Appendage (4.5×10⁻³²); Heart_Left_Ventricle (1.1×10⁻²¹); Pancreas (1.1×10⁻¹⁴); Testis (4×10⁻¹³); Artery_Aorta (4.7×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -21636,7 +21650,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>Artery_Tibial (1.3×10⁻²¹); Thyroid (2.1×10⁻¹⁶); Muscle_Skeletal (8.6×10⁻¹⁶); Nerve_Tibial (1.2×10⁻¹⁴); Cells_Cultured_fibroblasts (5.3×10⁻¹³); Esophagus_Muscularis (7.5×10⁻¹³); Prostate (1.6×10⁻⁰⁹); Brain_Cerebellum (2.2×10⁻⁰⁹); Artery_Aorta (3.5×10⁻⁰⁹); Brain_Hypothalamus (4.5×10⁻⁰⁸)</t>
+          <t>Artery_Tibial (1.3×10⁻²¹); Thyroid (2.1×10⁻¹⁶); Muscle_Skeletal (8.6×10⁻¹⁶); Nerve_Tibial (1.2×10⁻¹⁴); Cells_Cultured_fibroblasts (5.3×10⁻¹³); Esophagus_Muscularis (7.5×10⁻¹³); Prostate (1.6×10⁻⁹); Brain_Cerebellum (2.2×10⁻⁹); Artery_Aorta (3.5×10⁻⁹); Brain_Hypothalamus (4.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
@@ -21992,7 +22006,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (8.8×10⁻¹¹); Skin_Not_Sun_Exposed_Suprapubic (5.2×10⁻⁰⁹)</t>
+          <t>Cells_Cultured_fibroblasts (8.8×10⁻¹¹); Skin_Not_Sun_Exposed_Suprapubic (5.2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr"/>
@@ -22208,7 +22222,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>Esophagus_Muscularis (1.7×10⁻⁰⁹)</t>
+          <t>Esophagus_Muscularis (1.7×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -22312,7 +22326,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>Testis (3.3×10⁻²²); Pituitary (1.5×10⁻¹⁴); Ovary (1.9×10⁻¹¹); Nerve_Tibial (2.6×10⁻⁰⁹)</t>
+          <t>Testis (3.3×10⁻²²); Pituitary (1.5×10⁻¹⁴); Ovary (1.9×10⁻¹¹); Nerve_Tibial (2.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -22628,7 +22642,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (1.5×10⁻²²); Brain_Cerebellar_Hemisphere (1.5×10⁻¹⁶); Esophagus_Mucosa (1.1×10⁻¹³); Brain_Cortex (5.9×10⁻¹³); Nerve_Tibial (2.4×10⁻¹¹); Pancreas (4.9×10⁻⁰⁹)</t>
+          <t>Brain_Cerebellum (1.5×10⁻²²); Brain_Cerebellar_Hemisphere (1.5×10⁻¹⁶); Esophagus_Mucosa (1.1×10⁻¹³); Brain_Cortex (5.9×10⁻¹³); Nerve_Tibial (2.4×10⁻¹¹); Pancreas (4.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -22736,7 +22750,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (3.6×10⁻³³); Brain_Cerebellar_Hemisphere (8.4×10⁻²⁶); Lung (6.2×10⁻¹⁸); Esophagus_Mucosa (2×10⁻¹⁴); Spleen (2.4×10⁻¹²); Brain_Putamen_basal_ganglia (8.8×10⁻¹¹); Cells_Cultured_fibroblasts (3.6×10⁻⁰⁸); Breast_Mammary_Tissue (4.1×10⁻⁰⁸)</t>
+          <t>Brain_Cerebellum (3.6×10⁻³³); Brain_Cerebellar_Hemisphere (8.4×10⁻²⁶); Lung (6.2×10⁻¹⁸); Esophagus_Mucosa (2×10⁻¹⁴); Spleen (2.4×10⁻¹²); Brain_Putamen_basal_ganglia (8.8×10⁻¹¹); Cells_Cultured_fibroblasts (3.6×10⁻⁸); Breast_Mammary_Tissue (4.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -22840,7 +22854,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (9.8×10⁻¹¹); Lung (8.7×10⁻⁰⁹)</t>
+          <t>Cells_Cultured_fibroblasts (9.8×10⁻¹¹); Lung (8.7×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -22948,7 +22962,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>Skin_Not_Sun_Exposed_Suprapubic (2.7×10⁻²³); Skin_Sun_Exposed_Lower_leg (2.4×10⁻²⁰); Adipose_Subcutaneous (5.3×10⁻¹⁴); Esophagus_Mucosa (7.8×10⁻¹⁴); Cells_Cultured_fibroblasts (7.1×10⁻⁰⁹); Lung (1.2×10⁻⁰⁸)</t>
+          <t>Skin_Not_Sun_Exposed_Suprapubic (2.7×10⁻²³); Skin_Sun_Exposed_Lower_leg (2.4×10⁻²⁰); Adipose_Subcutaneous (5.3×10⁻¹⁴); Esophagus_Mucosa (7.8×10⁻¹⁴); Cells_Cultured_fibroblasts (7.1×10⁻⁹); Lung (1.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -23260,7 +23274,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (1.5×10⁻¹⁵); Skin_Not_Sun_Exposed_Suprapubic (3.5×10⁻¹⁵); Esophagus_Mucosa (1.5×10⁻¹¹); Adipose_Subcutaneous (3.2×10⁻¹⁰); Esophagus_Muscularis (6.5×10⁻¹⁰); Nerve_Tibial (1.1×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (1.5×10⁻¹⁵); Skin_Not_Sun_Exposed_Suprapubic (3.5×10⁻¹⁵); Esophagus_Mucosa (1.5×10⁻¹¹); Adipose_Subcutaneous (3.2×10⁻¹⁰); Esophagus_Muscularis (6.5×10⁻¹⁰); Nerve_Tibial (1.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -23364,7 +23378,7 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>Breast_Mammary_Tissue (4.7×10⁻²⁴); Adipose_Visceral_Omentum (1.3×10⁻²²); Adipose_Subcutaneous (5.4×10⁻¹⁸); Nerve_Tibial (4.1×10⁻¹⁴); Esophagus_Muscularis (2.5×10⁻¹⁰); Muscle_Skeletal (4.6×10⁻⁰⁸)</t>
+          <t>Breast_Mammary_Tissue (4.7×10⁻²⁴); Adipose_Visceral_Omentum (1.3×10⁻²²); Adipose_Subcutaneous (5.4×10⁻¹⁸); Nerve_Tibial (4.1×10⁻¹⁴); Esophagus_Muscularis (2.5×10⁻¹⁰); Muscle_Skeletal (4.6×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -23468,7 +23482,7 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>Spleen (1.3×10⁻¹⁸); Nerve_Tibial (1.7×10⁻¹⁰); Adipose_Subcutaneous (8.4×10⁻⁰⁹); Breast_Mammary_Tissue (1.3×10⁻⁰⁸)</t>
+          <t>Spleen (1.3×10⁻¹⁸); Nerve_Tibial (1.7×10⁻¹⁰); Adipose_Subcutaneous (8.4×10⁻⁹); Breast_Mammary_Tissue (1.3×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -23676,7 +23690,7 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>Adipose_Visceral_Omentum (8.9×10⁻¹²); Adipose_Subcutaneous (4.1×10⁻⁰⁸)</t>
+          <t>Adipose_Visceral_Omentum (8.9×10⁻¹²); Adipose_Subcutaneous (4.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -23780,7 +23794,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>Esophagus_Muscularis (1.1×10⁻¹⁴); Adipose_Subcutaneous (9.5×10⁻¹¹); Esophagus_Gastroesophageal_Junction (7.1×10⁻¹⁰); Stomach (9.6×10⁻⁰⁹)</t>
+          <t>Esophagus_Muscularis (1.1×10⁻¹⁴); Adipose_Subcutaneous (9.5×10⁻¹¹); Esophagus_Gastroesophageal_Junction (7.1×10⁻¹⁰); Stomach (9.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -23992,7 +24006,7 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>Esophagus_Mucosa (7.4×10⁻¹⁷); Skin_Not_Sun_Exposed_Suprapubic (3.2×10⁻¹⁰); Testis (1.4×10⁻⁰⁹)</t>
+          <t>Esophagus_Mucosa (7.4×10⁻¹⁷); Skin_Not_Sun_Exposed_Suprapubic (3.2×10⁻¹⁰); Testis (1.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -24100,7 +24114,7 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>Esophagus_Muscularis (4×10⁻⁰⁸)</t>
+          <t>Esophagus_Muscularis (4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -24204,7 +24218,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (5.2×10⁻¹⁰); Muscle_Skeletal (1.1×10⁻⁰⁹); Nerve_Tibial (1.9×10⁻⁰⁹)</t>
+          <t>Cells_Cultured_fibroblasts (5.2×10⁻¹⁰); Muscle_Skeletal (1.1×10⁻⁹); Nerve_Tibial (1.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -24516,7 +24530,7 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (1.6×10⁻¹⁰); Cells_Cultured_fibroblasts (3.4×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (1.6×10⁻¹⁰); Cells_Cultured_fibroblasts (3.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -24828,7 +24842,7 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (3.7×10⁻⁵⁴); Spleen (5×10⁻²⁴); Lung (5.7×10⁻¹⁸); Colon_Sigmoid (1×10⁻¹³); Adipose_Subcutaneous (1.5×10⁻¹²); Esophagus_Muscularis (3.3×10⁻¹⁰); Esophagus_Gastroesophageal_Junction (6.7×10⁻¹⁰); Adipose_Visceral_Omentum (1.7×10⁻⁰⁸); Skin_Not_Sun_Exposed_Suprapubic (2.7×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (3.7×10⁻⁵⁴); Spleen (5×10⁻²⁴); Lung (5.7×10⁻¹⁸); Colon_Sigmoid (1×10⁻¹³); Adipose_Subcutaneous (1.5×10⁻¹²); Esophagus_Muscularis (3.3×10⁻¹⁰); Esophagus_Gastroesophageal_Junction (6.7×10⁻¹⁰); Adipose_Visceral_Omentum (1.7×10⁻⁸); Skin_Not_Sun_Exposed_Suprapubic (2.7×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q183" t="inlineStr"/>
@@ -25056,7 +25070,7 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>Testis (4.8×10⁻⁰⁹)</t>
+          <t>Testis (4.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q185" t="inlineStr"/>
@@ -25264,7 +25278,7 @@
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (4.9×10⁻²²); Brain_Cerebellar_Hemisphere (1.1×10⁻¹¹); Pancreas (4.4×10⁻⁰⁹)</t>
+          <t>Brain_Cerebellum (4.9×10⁻²²); Brain_Cerebellar_Hemisphere (1.1×10⁻¹¹); Pancreas (4.4×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q187" t="inlineStr"/>
@@ -25372,7 +25386,7 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>Esophagus_Mucosa (8.1×10⁻⁴²); Cells_Cultured_fibroblasts (4.2×10⁻⁰⁸)</t>
+          <t>Esophagus_Mucosa (8.1×10⁻⁴²); Cells_Cultured_fibroblasts (4.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q188" t="inlineStr"/>
@@ -25476,7 +25490,7 @@
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (7.2×10⁻⁰⁹)</t>
+          <t>Brain_Cerebellum (7.2×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q189" t="inlineStr"/>
@@ -26636,7 +26650,7 @@
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>Small_Intestine_Terminal_Ileum (4.1×10⁻¹⁷); Brain_Cerebellum (6.7×10⁻⁰⁹); Brain_Cerebellar_Hemisphere (6.8×10⁻⁰⁹); Nerve_Tibial (2.8×10⁻⁰⁸); Colon_Transverse (2.9×10⁻⁰⁸); Brain_Caudate_basal_ganglia (3.5×10⁻⁰⁸)</t>
+          <t>Small_Intestine_Terminal_Ileum (4.1×10⁻¹⁷); Brain_Cerebellum (6.7×10⁻⁹); Brain_Cerebellar_Hemisphere (6.8×10⁻⁹); Nerve_Tibial (2.8×10⁻⁸); Colon_Transverse (2.9×10⁻⁸); Brain_Caudate_basal_ganglia (3.5×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q200" t="inlineStr"/>
@@ -26952,7 +26966,7 @@
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>Esophagus_Gastroesophageal_Junction (4.5×10⁻⁰⁹); Colon_Sigmoid (6.8×10⁻⁰⁹)</t>
+          <t>Esophagus_Gastroesophageal_Junction (4.5×10⁻⁹); Colon_Sigmoid (6.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q203" t="inlineStr"/>
@@ -27056,7 +27070,7 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>Brain_Caudate_basal_ganglia (6.2×10⁻²⁸); Brain_Cortex (2.2×10⁻²²); Brain_Putamen_basal_ganglia (3×10⁻²¹); Brain_Spinal_cord_cervical_c-1 (1.5×10⁻²⁰); Brain_Substantia_nigra (1.7×10⁻¹⁸); Brain_Hippocampus (4.6×10⁻¹⁶); Brain_Amygdala (3.6×10⁻¹⁵); Brain_Hypothalamus (6.6×10⁻⁰⁹); Brain_Anterior_cingulate_cortex_BA24 (8.3×10⁻⁰⁹); Brain_Frontal_Cortex_BA9 (3.1×10⁻⁰⁸)</t>
+          <t>Brain_Caudate_basal_ganglia (6.2×10⁻²⁸); Brain_Cortex (2.2×10⁻²²); Brain_Putamen_basal_ganglia (3×10⁻²¹); Brain_Spinal_cord_cervical_c-1 (1.5×10⁻²⁰); Brain_Substantia_nigra (1.7×10⁻¹⁸); Brain_Hippocampus (4.6×10⁻¹⁶); Brain_Amygdala (3.6×10⁻¹⁵); Brain_Hypothalamus (6.6×10⁻⁹); Brain_Anterior_cingulate_cortex_BA24 (8.3×10⁻⁹); Brain_Frontal_Cortex_BA9 (3.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q204" t="inlineStr"/>
@@ -27160,7 +27174,7 @@
       </c>
       <c r="P205" t="inlineStr">
         <is>
-          <t>Skin_Not_Sun_Exposed_Suprapubic (4.8×10⁻²⁹); Skin_Sun_Exposed_Lower_leg (1.2×10⁻¹⁹); Colon_Transverse (2.9×10⁻⁰⁹)</t>
+          <t>Skin_Not_Sun_Exposed_Suprapubic (4.8×10⁻²⁹); Skin_Sun_Exposed_Lower_leg (1.2×10⁻¹⁹); Colon_Transverse (2.9×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q205" t="inlineStr"/>
@@ -27264,7 +27278,7 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (9.7×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (4.2×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (9.7×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (4.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q206" t="inlineStr"/>
@@ -27472,7 +27486,7 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>Testis (4.5×10⁻⁰⁹)</t>
+          <t>Testis (4.5×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q208" t="inlineStr"/>
@@ -27680,7 +27694,7 @@
       </c>
       <c r="P210" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (5.4×10⁻⁶⁶); Skin_Not_Sun_Exposed_Suprapubic (8.2×10⁻⁴¹); Brain_Frontal_Cortex_BA9 (2.5×10⁻¹²); Adipose_Subcutaneous (2×10⁻¹⁰); Brain_Cortex (1.4×10⁻⁰⁹); Minor_Salivary_Gland (1.2×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (5.4×10⁻⁶⁶); Skin_Not_Sun_Exposed_Suprapubic (8.2×10⁻⁴¹); Brain_Frontal_Cortex_BA9 (2.5×10⁻¹²); Adipose_Subcutaneous (2×10⁻¹⁰); Brain_Cortex (1.4×10⁻⁹); Minor_Salivary_Gland (1.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q210" t="inlineStr"/>
@@ -28100,7 +28114,7 @@
       </c>
       <c r="P214" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (4.9×10⁻¹¹); Muscle_Skeletal (1.3×10⁻¹⁰); Adipose_Subcutaneous (2.3×10⁻¹⁰); Colon_Sigmoid (1.1×10⁻⁰⁸); Testis (1.4×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (4.9×10⁻¹¹); Muscle_Skeletal (1.3×10⁻¹⁰); Adipose_Subcutaneous (2.3×10⁻¹⁰); Colon_Sigmoid (1.1×10⁻⁸); Testis (1.4×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q214" t="inlineStr"/>
@@ -28416,7 +28430,7 @@
       </c>
       <c r="P217" t="inlineStr">
         <is>
-          <t>Thyroid (8.5×10⁻¹⁸); Spleen (4.7×10⁻¹⁴); Nerve_Tibial (1.8×10⁻⁰⁹)</t>
+          <t>Thyroid (8.5×10⁻¹⁸); Spleen (4.7×10⁻¹⁴); Nerve_Tibial (1.8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q217" t="inlineStr"/>
@@ -28520,7 +28534,7 @@
       </c>
       <c r="P218" t="inlineStr">
         <is>
-          <t>Cells_Cultured_fibroblasts (1.2×10⁻⁰⁸); Testis (1.8×10⁻⁰⁸)</t>
+          <t>Cells_Cultured_fibroblasts (1.2×10⁻⁸); Testis (1.8×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q218" t="inlineStr"/>
@@ -28624,7 +28638,7 @@
       </c>
       <c r="P219" t="inlineStr">
         <is>
-          <t>Testis (2.6×10⁻⁰⁹)</t>
+          <t>Testis (2.6×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q219" t="inlineStr"/>
@@ -28728,7 +28742,7 @@
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>Brain_Cerebellum (8.6×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (8.8×10⁻¹⁰); Brain_Cerebellar_Hemisphere (8×10⁻⁰⁹)</t>
+          <t>Brain_Cerebellum (8.6×10⁻¹²); Brain_Nucleus_accumbens_basal_ganglia (8.8×10⁻¹⁰); Brain_Cerebellar_Hemisphere (8×10⁻⁹)</t>
         </is>
       </c>
       <c r="Q220" t="inlineStr"/>
@@ -28944,7 +28958,7 @@
       </c>
       <c r="P222" t="inlineStr">
         <is>
-          <t>Nerve_Tibial (4.1×10⁻⁰⁸)</t>
+          <t>Nerve_Tibial (4.1×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q222" t="inlineStr"/>
@@ -29048,7 +29062,7 @@
       </c>
       <c r="P223" t="inlineStr">
         <is>
-          <t>Skin_Sun_Exposed_Lower_leg (5.9×10⁻¹⁵); Esophagus_Mucosa (1.2×10⁻⁰⁸); Testis (4.2×10⁻⁰⁸)</t>
+          <t>Skin_Sun_Exposed_Lower_leg (5.9×10⁻¹⁵); Esophagus_Mucosa (1.2×10⁻⁸); Testis (4.2×10⁻⁸)</t>
         </is>
       </c>
       <c r="Q223" t="inlineStr"/>
@@ -35249,7 +35263,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Cultured fibroblasts (8.8×10⁻¹¹; n=483); Skin Not Sun Exposed Suprapubic (5.2×10⁻⁰⁹; n=517)</t>
+          <t>Cultured fibroblasts (8.8×10⁻¹¹; n=483); Skin Not Sun Exposed Suprapubic (5.2×10⁻⁹; n=517)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -35323,7 +35337,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Esophagus Muscularis (1.7×10⁻⁰⁹; n=465)</t>
+          <t>Esophagus Muscularis (1.7×10⁻⁹; n=465)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -35360,7 +35374,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Testis (3.3×10⁻²²; n=322); Pituitary (1.5×10⁻¹⁴; n=237); Ovary (1.9×10⁻¹¹; n=167); Nerve Tibial (2.6×10⁻⁰⁹; n=532)</t>
+          <t>Testis (3.3×10⁻²²; n=322); Pituitary (1.5×10⁻¹⁴; n=237); Ovary (1.9×10⁻¹¹; n=167); Nerve Tibial (2.6×10⁻⁹; n=532)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -35471,7 +35485,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Brain Cerebellum (1.5×10⁻²²; n=209); Brain Cerebellar Hemisphere (1.5×10⁻¹⁶; n=175); Esophagus Mucosa (1.1×10⁻¹³; n=497); Brain Cortex (5.9×10⁻¹³; n=205); Nerve Tibial (2.4×10⁻¹¹; n=532); Pancreas (4.9×10⁻⁰⁹; n=305)</t>
+          <t>Brain Cerebellum (1.5×10⁻²²; n=209); Brain Cerebellar Hemisphere (1.5×10⁻¹⁶; n=175); Esophagus Mucosa (1.1×10⁻¹³; n=497); Brain Cortex (5.9×10⁻¹³; n=205); Nerve Tibial (2.4×10⁻¹¹; n=532); Pancreas (4.9×10⁻⁹; n=305)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -35508,7 +35522,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Brain Cerebellum (3.6×10⁻³³; n=209); Brain Cerebellar Hemisphere (8.4×10⁻²⁶; n=175); Lung (6.2×10⁻¹⁸; n=515); Esophagus Mucosa (2×10⁻¹⁴; n=497); Spleen (2.4×10⁻¹²; n=227); Brain Putamen basal ganglia (8.8×10⁻¹¹; n=170); Cultured fibroblasts (3.6×10⁻⁰⁸; n=483); Breast Mammary Tissue (4.1×10⁻⁰⁸; n=396)</t>
+          <t>Brain Cerebellum (3.6×10⁻³³; n=209); Brain Cerebellar Hemisphere (8.4×10⁻²⁶; n=175); Lung (6.2×10⁻¹⁸; n=515); Esophagus Mucosa (2×10⁻¹⁴; n=497); Spleen (2.4×10⁻¹²; n=227); Brain Putamen basal ganglia (8.8×10⁻¹¹; n=170); Cultured fibroblasts (3.6×10⁻⁸; n=483); Breast Mammary Tissue (4.1×10⁻⁸; n=396)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -35545,7 +35559,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Cultured fibroblasts (9.8×10⁻¹¹; n=483); Lung (8.7×10⁻⁰⁹; n=515)</t>
+          <t>Cultured fibroblasts (9.8×10⁻¹¹; n=483); Lung (8.7×10⁻⁹; n=515)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -35582,7 +35596,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Skin Not Sun Exposed Suprapubic (2.7×10⁻²³; n=517); Skin Sun Exposed Lower leg (2.4×10⁻²⁰; n=605); Adipose Subcutaneous (5.3×10⁻¹⁴; n=581); Esophagus Mucosa (7.8×10⁻¹⁴; n=497); Cultured fibroblasts (7.1×10⁻⁰⁹; n=483); Lung (1.2×10⁻⁰⁸; n=515)</t>
+          <t>Skin Not Sun Exposed Suprapubic (2.7×10⁻²³; n=517); Skin Sun Exposed Lower leg (2.4×10⁻²⁰; n=605); Adipose Subcutaneous (5.3×10⁻¹⁴; n=581); Esophagus Mucosa (7.8×10⁻¹⁴; n=497); Cultured fibroblasts (7.1×10⁻⁹; n=483); Lung (1.2×10⁻⁸; n=515)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -35693,7 +35707,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Skin Sun Exposed Lower leg (1.5×10⁻¹⁵; n=605); Skin Not Sun Exposed Suprapubic (3.5×10⁻¹⁵; n=517); Esophagus Mucosa (1.5×10⁻¹¹; n=497); Adipose Subcutaneous (3.2×10⁻¹⁰; n=581); Esophagus Muscularis (6.5×10⁻¹⁰; n=465); Nerve Tibial (1.1×10⁻⁰⁸; n=532)</t>
+          <t>Skin Sun Exposed Lower leg (1.5×10⁻¹⁵; n=605); Skin Not Sun Exposed Suprapubic (3.5×10⁻¹⁵; n=517); Esophagus Mucosa (1.5×10⁻¹¹; n=497); Adipose Subcutaneous (3.2×10⁻¹⁰; n=581); Esophagus Muscularis (6.5×10⁻¹⁰; n=465); Nerve Tibial (1.1×10⁻⁸; n=532)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -35730,7 +35744,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Breast Mammary Tissue (4.7×10⁻²⁴; n=396); Adipose Visceral Omentum (1.3×10⁻²²; n=469); Adipose Subcutaneous (5.4×10⁻¹⁸; n=581); Nerve Tibial (4.1×10⁻¹⁴; n=532); Esophagus Muscularis (2.5×10⁻¹⁰; n=465); Muscle Skeletal (4.6×10⁻⁰⁸; n=706)</t>
+          <t>Breast Mammary Tissue (4.7×10⁻²⁴; n=396); Adipose Visceral Omentum (1.3×10⁻²²; n=469); Adipose Subcutaneous (5.4×10⁻¹⁸; n=581); Nerve Tibial (4.1×10⁻¹⁴; n=532); Esophagus Muscularis (2.5×10⁻¹⁰; n=465); Muscle Skeletal (4.6×10⁻⁸; n=706)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -35767,7 +35781,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Spleen (1.3×10⁻¹⁸; n=227); Nerve Tibial (1.7×10⁻¹⁰; n=532); Adipose Subcutaneous (8.4×10⁻⁰⁹; n=581); Breast Mammary Tissue (1.3×10⁻⁰⁸; n=396)</t>
+          <t>Spleen (1.3×10⁻¹⁸; n=227); Nerve Tibial (1.7×10⁻¹⁰; n=532); Adipose Subcutaneous (8.4×10⁻⁹; n=581); Breast Mammary Tissue (1.3×10⁻⁸; n=396)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -35841,7 +35855,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Adipose Visceral Omentum (8.9×10⁻¹²; n=469); Adipose Subcutaneous (4.1×10⁻⁰⁸; n=581)</t>
+          <t>Adipose Visceral Omentum (8.9×10⁻¹²; n=469); Adipose Subcutaneous (4.1×10⁻⁸; n=581)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -35878,7 +35892,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Esophagus Muscularis (1.1×10⁻¹⁴; n=465); Adipose Subcutaneous (9.5×10⁻¹¹; n=581); Esophagus Gastroesophageal Junction (7.1×10⁻¹⁰; n=330); Stomach (9.6×10⁻⁰⁹; n=324)</t>
+          <t>Esophagus Muscularis (1.1×10⁻¹⁴; n=465); Adipose Subcutaneous (9.5×10⁻¹¹; n=581); Esophagus Gastroesophageal Junction (7.1×10⁻¹⁰; n=330); Stomach (9.6×10⁻⁹; n=324)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -35952,7 +35966,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Esophagus Mucosa (7.4×10⁻¹⁷; n=497); Skin Not Sun Exposed Suprapubic (3.2×10⁻¹⁰; n=517); Testis (1.4×10⁻⁰⁹; n=322)</t>
+          <t>Esophagus Mucosa (7.4×10⁻¹⁷; n=497); Skin Not Sun Exposed Suprapubic (3.2×10⁻¹⁰; n=517); Testis (1.4×10⁻⁹; n=322)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -35989,7 +36003,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Esophagus Muscularis (4×10⁻⁰⁸; n=465)</t>
+          <t>Esophagus Muscularis (4×10⁻⁸; n=465)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -36026,7 +36040,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Cultured fibroblasts (5.2×10⁻¹⁰; n=483); Muscle Skeletal (1.1×10⁻⁰⁹; n=706); Nerve Tibial (1.9×10⁻⁰⁹; n=532)</t>
+          <t>Cultured fibroblasts (5.2×10⁻¹⁰; n=483); Muscle Skeletal (1.1×10⁻⁹; n=706); Nerve Tibial (1.9×10⁻⁹; n=532)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -36137,7 +36151,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Nerve Tibial (1.6×10⁻¹⁰; n=532); Cultured fibroblasts (3.4×10⁻⁰⁸; n=483)</t>
+          <t>Nerve Tibial (1.6×10⁻¹⁰; n=532); Cultured fibroblasts (3.4×10⁻⁸; n=483)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -36248,7 +36262,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Nerve Tibial (3.7×10⁻⁵⁴; n=532); Spleen (5×10⁻²⁴; n=227); Lung (5.7×10⁻¹⁸; n=515); Colon Sigmoid (1×10⁻¹³; n=318); Adipose Subcutaneous (1.5×10⁻¹²; n=581); Esophagus Muscularis (3.3×10⁻¹⁰; n=465); Esophagus Gastroesophageal Junction (6.7×10⁻¹⁰; n=330); Adipose Visceral Omentum (1.7×10⁻⁰⁸; n=469); Skin Not Sun Exposed Suprapubic (2.7×10⁻⁰⁸; n=517)</t>
+          <t>Nerve Tibial (3.7×10⁻⁵⁴; n=532); Spleen (5×10⁻²⁴; n=227); Lung (5.7×10⁻¹⁸; n=515); Colon Sigmoid (1×10⁻¹³; n=318); Adipose Subcutaneous (1.5×10⁻¹²; n=581); Esophagus Muscularis (3.3×10⁻¹⁰; n=465); Esophagus Gastroesophageal Junction (6.7×10⁻¹⁰; n=330); Adipose Visceral Omentum (1.7×10⁻⁸; n=469); Skin Not Sun Exposed Suprapubic (2.7×10⁻⁸; n=517)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -36322,7 +36336,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Testis (4.8×10⁻⁰⁹; n=322)</t>
+          <t>Testis (4.8×10⁻⁹; n=322)</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -36396,7 +36410,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Brain Cerebellum (4.9×10⁻²²; n=209); Brain Cerebellar Hemisphere (1.1×10⁻¹¹; n=175); Pancreas (4.4×10⁻⁰⁹; n=305)</t>
+          <t>Brain Cerebellum (4.9×10⁻²²; n=209); Brain Cerebellar Hemisphere (1.1×10⁻¹¹; n=175); Pancreas (4.4×10⁻⁹; n=305)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -36433,7 +36447,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Esophagus Mucosa (8.1×10⁻⁴²; n=497); Cultured fibroblasts (4.2×10⁻⁰⁸; n=483)</t>
+          <t>Esophagus Mucosa (8.1×10⁻⁴²; n=497); Cultured fibroblasts (4.2×10⁻⁸; n=483)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -36470,7 +36484,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Brain Cerebellum (7.2×10⁻⁰⁹; n=209)</t>
+          <t>Brain Cerebellum (7.2×10⁻⁹; n=209)</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -36877,7 +36891,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Small Intestine Terminal Ileum (4.1×10⁻¹⁷; n=174); Brain Cerebellum (6.7×10⁻⁰⁹; n=209); Brain Cerebellar Hemisphere (6.8×10⁻⁰⁹; n=175); Nerve Tibial (2.8×10⁻⁰⁸; n=532); Colon Transverse (2.9×10⁻⁰⁸; n=368); Brain Caudate basal ganglia (3.5×10⁻⁰⁸; n=194)</t>
+          <t>Small Intestine Terminal Ileum (4.1×10⁻¹⁷; n=174); Brain Cerebellum (6.7×10⁻⁹; n=209); Brain Cerebellar Hemisphere (6.8×10⁻⁹; n=175); Nerve Tibial (2.8×10⁻⁸; n=532); Colon Transverse (2.9×10⁻⁸; n=368); Brain Caudate basal ganglia (3.5×10⁻⁸; n=194)</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -36988,7 +37002,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Esophagus Gastroesophageal Junction (4.5×10⁻⁰⁹; n=330); Colon Sigmoid (6.8×10⁻⁰⁹; n=318)</t>
+          <t>Esophagus Gastroesophageal Junction (4.5×10⁻⁹; n=330); Colon Sigmoid (6.8×10⁻⁹; n=318)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -37025,7 +37039,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Brain Caudate basal ganglia (6.2×10⁻²⁸; n=194); Brain Cortex (2.2×10⁻²²; n=205); Brain Putamen basal ganglia (3×10⁻²¹; n=170); Brain Spinal cord cervical c-1 (1.5×10⁻²⁰; n=126); Brain Substantia nigra (1.7×10⁻¹⁸; n=114); Brain Hippocampus (4.6×10⁻¹⁶; n=165); Brain Amygdala (3.6×10⁻¹⁵; n=129); Brain Hypothalamus (6.6×10⁻⁰⁹; n=170); Brain Anterior cingulate cortex BA24 (8.3×10⁻⁰⁹; n=147); Brain Frontal Cortex BA9 (3.1×10⁻⁰⁸; n=175)</t>
+          <t>Brain Caudate basal ganglia (6.2×10⁻²⁸; n=194); Brain Cortex (2.2×10⁻²²; n=205); Brain Putamen basal ganglia (3×10⁻²¹; n=170); Brain Spinal cord cervical c-1 (1.5×10⁻²⁰; n=126); Brain Substantia nigra (1.7×10⁻¹⁸; n=114); Brain Hippocampus (4.6×10⁻¹⁶; n=165); Brain Amygdala (3.6×10⁻¹⁵; n=129); Brain Hypothalamus (6.6×10⁻⁹; n=170); Brain Anterior cingulate cortex BA24 (8.3×10⁻⁹; n=147); Brain Frontal Cortex BA9 (3.1×10⁻⁸; n=175)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -37062,7 +37076,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Skin Not Sun Exposed Suprapubic (4.8×10⁻²⁹; n=517); Skin Sun Exposed Lower leg (1.2×10⁻¹⁹; n=605); Colon Transverse (2.9×10⁻⁰⁹; n=368)</t>
+          <t>Skin Not Sun Exposed Suprapubic (4.8×10⁻²⁹; n=517); Skin Sun Exposed Lower leg (1.2×10⁻¹⁹; n=605); Colon Transverse (2.9×10⁻⁹; n=368)</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -37099,7 +37113,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Nerve Tibial (9.7×10⁻¹²; n=532); Brain Nucleus accumbens basal ganglia (4.2×10⁻⁰⁸; n=202)</t>
+          <t>Nerve Tibial (9.7×10⁻¹²; n=532); Brain Nucleus accumbens basal ganglia (4.2×10⁻⁸; n=202)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -37173,7 +37187,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Testis (4.5×10⁻⁰⁹; n=322)</t>
+          <t>Testis (4.5×10⁻⁹; n=322)</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -37247,7 +37261,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Skin Sun Exposed Lower leg (5.4×10⁻⁶⁶; n=605); Skin Not Sun Exposed Suprapubic (8.2×10⁻⁴¹; n=517); Brain Frontal Cortex BA9 (2.5×10⁻¹²; n=175); Adipose Subcutaneous (2×10⁻¹⁰; n=581); Brain Cortex (1.4×10⁻⁰⁹; n=205); Minor Salivary Gland (1.2×10⁻⁰⁸; n=144)</t>
+          <t>Skin Sun Exposed Lower leg (5.4×10⁻⁶⁶; n=605); Skin Not Sun Exposed Suprapubic (8.2×10⁻⁴¹; n=517); Brain Frontal Cortex BA9 (2.5×10⁻¹²; n=175); Adipose Subcutaneous (2×10⁻¹⁰; n=581); Brain Cortex (1.4×10⁻⁹; n=205); Minor Salivary Gland (1.2×10⁻⁸; n=144)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -37395,7 +37409,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Nerve Tibial (4.9×10⁻¹¹; n=532); Muscle Skeletal (1.3×10⁻¹⁰; n=706); Adipose Subcutaneous (2.3×10⁻¹⁰; n=581); Colon Sigmoid (1.1×10⁻⁰⁸; n=318); Testis (1.4×10⁻⁰⁸; n=322)</t>
+          <t>Nerve Tibial (4.9×10⁻¹¹; n=532); Muscle Skeletal (1.3×10⁻¹⁰; n=706); Adipose Subcutaneous (2.3×10⁻¹⁰; n=581); Colon Sigmoid (1.1×10⁻⁸; n=318); Testis (1.4×10⁻⁸; n=322)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -37506,7 +37520,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Thyroid (8.5×10⁻¹⁸; n=574); Spleen (4.7×10⁻¹⁴; n=227); Nerve Tibial (1.8×10⁻⁰⁹; n=532)</t>
+          <t>Thyroid (8.5×10⁻¹⁸; n=574); Spleen (4.7×10⁻¹⁴; n=227); Nerve Tibial (1.8×10⁻⁹; n=532)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -37543,7 +37557,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Cultured fibroblasts (1.2×10⁻⁰⁸; n=483); Testis (1.8×10⁻⁰⁸; n=322)</t>
+          <t>Cultured fibroblasts (1.2×10⁻⁸; n=483); Testis (1.8×10⁻⁸; n=322)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -37580,7 +37594,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Testis (2.6×10⁻⁰⁹; n=322)</t>
+          <t>Testis (2.6×10⁻⁹; n=322)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -37617,7 +37631,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Brain Cerebellum (8.6×10⁻¹²; n=209); Brain Nucleus accumbens basal ganglia (8.8×10⁻¹⁰; n=202); Brain Cerebellar Hemisphere (8×10⁻⁰⁹; n=175)</t>
+          <t>Brain Cerebellum (8.6×10⁻¹²; n=209); Brain Nucleus accumbens basal ganglia (8.8×10⁻¹⁰; n=202); Brain Cerebellar Hemisphere (8×10⁻⁹; n=175)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -37691,7 +37705,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Nerve Tibial (4.1×10⁻⁰⁸; n=532)</t>
+          <t>Nerve Tibial (4.1×10⁻⁸; n=532)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -37728,7 +37742,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Skin Sun Exposed Lower leg (5.9×10⁻¹⁵; n=605); Esophagus Mucosa (1.2×10⁻⁰⁸; n=497); Testis (4.2×10⁻⁰⁸; n=322)</t>
+          <t>Skin Sun Exposed Lower leg (5.9×10⁻¹⁵; n=605); Esophagus Mucosa (1.2×10⁻⁸; n=497); Testis (4.2×10⁻⁸; n=322)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">

</xml_diff>